<commit_message>
Update: GEC template timesheet Single 08.08.2025.xlsx
</commit_message>
<xml_diff>
--- a/Samples/GEC template timesheet Single 08.08.2025.xlsx
+++ b/Samples/GEC template timesheet Single 08.08.2025.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="S:\HR ESSA\01. PAYROLL 2025\7. GEC PAYROLL 2025\GEC Payroll Automation project\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Projects\GEC\Samples\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{66388D80-D3BB-43F3-B42E-95C314B77B4D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C6FE9393-97AD-4660-A50B-A2B6AA319200}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="836" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" tabRatio="836" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Monthly Timesheet" sheetId="51" r:id="rId1"/>
@@ -20,16 +20,6 @@
     <definedName name="_xlnm.Print_Area" localSheetId="0">'Monthly Timesheet'!$A$1:$AJ$44</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
-  <extLst>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
 </workbook>
 </file>
 
@@ -129,13 +119,13 @@
     <t>Sun</t>
   </si>
   <si>
-    <t>Employee B</t>
-  </si>
-  <si>
     <t>Gabon</t>
   </si>
   <si>
     <t>Spain</t>
+  </si>
+  <si>
+    <t>Dummy Name 1</t>
   </si>
 </sst>
 </file>
@@ -1226,6 +1216,293 @@
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="16" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="6" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="6" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="6" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="35" fillId="0" borderId="35" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="36" fillId="0" borderId="33" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="36" fillId="0" borderId="36" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="41" xfId="1" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="2" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="2" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="2" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="2" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="2" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="29" xfId="1" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="165" fontId="34" fillId="0" borderId="41" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="165" fontId="34" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="45" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="4" borderId="42" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="4" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="4" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="46" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="2" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="2" borderId="48" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="5" borderId="46" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="5" borderId="47" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="7" borderId="42" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="7" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="7" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="7" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="7" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="7" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="49" fontId="21" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="21" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="21" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="5" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="5" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="5" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="26" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="26" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="26" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="7" borderId="43" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="7" borderId="44" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="16" fillId="5" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="16" fillId="5" borderId="44" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="21" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="21" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
+      <protection locked="0"/>
+    </xf>
     <xf numFmtId="0" fontId="16" fillId="2" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -1253,293 +1530,6 @@
       <protection locked="0"/>
     </xf>
     <xf numFmtId="165" fontId="21" fillId="0" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="49" fontId="21" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="21" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="5" borderId="46" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="5" borderId="47" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="7" borderId="42" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="7" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="7" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="7" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="7" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="7" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="49" fontId="21" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="49" fontId="21" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="49" fontId="21" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="5" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="5" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="5" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="26" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="26" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="26" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="7" borderId="43" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="7" borderId="44" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="16" fillId="5" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="16" fillId="5" borderId="44" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="45" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="4" borderId="42" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="4" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="4" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="46" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="2" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="2" borderId="48" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="6" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="6" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="6" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="35" fillId="0" borderId="35" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="49" fontId="36" fillId="0" borderId="33" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="49" fontId="36" fillId="0" borderId="36" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="0" borderId="41" xfId="1" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="2" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="2" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="2" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="2" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="2" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="0" borderId="29" xfId="1" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="165" fontId="34" fillId="0" borderId="41" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="165" fontId="34" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="16" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
@@ -3651,19 +3641,19 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:BA83"/>
-  <sheetFormatPr defaultColWidth="4.140625" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="4.1796875" defaultRowHeight="13" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="7.5703125" style="7" customWidth="1"/>
-    <col min="2" max="2" width="19.28515625" style="7" customWidth="1"/>
-    <col min="3" max="3" width="23.7109375" style="7" customWidth="1"/>
-    <col min="4" max="34" width="7.140625" style="7" customWidth="1"/>
-    <col min="35" max="35" width="17.28515625" style="7" customWidth="1"/>
-    <col min="36" max="36" width="16.28515625" style="7" customWidth="1"/>
-    <col min="37" max="38" width="6.140625" style="7" customWidth="1"/>
-    <col min="39" max="16384" width="4.140625" style="7"/>
+    <col min="1" max="1" width="7.54296875" style="7" customWidth="1"/>
+    <col min="2" max="2" width="19.26953125" style="7" customWidth="1"/>
+    <col min="3" max="3" width="23.7265625" style="7" customWidth="1"/>
+    <col min="4" max="34" width="7.1796875" style="7" customWidth="1"/>
+    <col min="35" max="35" width="17.26953125" style="7" customWidth="1"/>
+    <col min="36" max="36" width="16.26953125" style="7" customWidth="1"/>
+    <col min="37" max="38" width="6.1796875" style="7" customWidth="1"/>
+    <col min="39" max="16384" width="4.1796875" style="7"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:53" ht="39.75" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:53" ht="39.75" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A1" s="5" t="s">
         <v>24</v>
       </c>
@@ -3700,7 +3690,7 @@
       <c r="AN1" s="8"/>
       <c r="AO1" s="8"/>
     </row>
-    <row r="2" spans="1:53" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:53" ht="24.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A2" s="9" t="s">
         <v>17</v>
       </c>
@@ -3737,7 +3727,7 @@
       <c r="AN2" s="10"/>
       <c r="AO2" s="10"/>
     </row>
-    <row r="3" spans="1:53" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:53" ht="24.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A3" s="9"/>
       <c r="B3" s="6"/>
       <c r="C3" s="6"/>
@@ -3772,7 +3762,7 @@
       <c r="AN3" s="10"/>
       <c r="AO3" s="10"/>
     </row>
-    <row r="4" spans="1:53" ht="36" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:53" ht="36" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A4" s="9"/>
       <c r="B4" s="6"/>
       <c r="C4" s="6"/>
@@ -3807,47 +3797,47 @@
       <c r="AN4" s="10"/>
       <c r="AO4" s="10"/>
     </row>
-    <row r="5" spans="1:53" s="14" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A5" s="92" t="s">
+    <row r="5" spans="1:53" s="14" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.6">
+      <c r="A5" s="123" t="s">
         <v>14</v>
       </c>
-      <c r="B5" s="92"/>
-      <c r="C5" s="93"/>
-      <c r="D5" s="118" t="s">
-        <v>31</v>
-      </c>
-      <c r="E5" s="119"/>
-      <c r="F5" s="119"/>
-      <c r="G5" s="119"/>
-      <c r="H5" s="119"/>
-      <c r="I5" s="119"/>
-      <c r="J5" s="119"/>
-      <c r="K5" s="119"/>
-      <c r="L5" s="119"/>
-      <c r="M5" s="120"/>
+      <c r="B5" s="123"/>
+      <c r="C5" s="124"/>
+      <c r="D5" s="149" t="s">
+        <v>33</v>
+      </c>
+      <c r="E5" s="150"/>
+      <c r="F5" s="150"/>
+      <c r="G5" s="150"/>
+      <c r="H5" s="150"/>
+      <c r="I5" s="150"/>
+      <c r="J5" s="150"/>
+      <c r="K5" s="150"/>
+      <c r="L5" s="150"/>
+      <c r="M5" s="151"/>
       <c r="N5" s="54"/>
       <c r="O5" s="54"/>
       <c r="P5" s="54"/>
-      <c r="Q5" s="102" t="s">
+      <c r="Q5" s="133" t="s">
         <v>15</v>
       </c>
-      <c r="R5" s="102"/>
-      <c r="S5" s="102"/>
-      <c r="T5" s="102"/>
+      <c r="R5" s="133"/>
+      <c r="S5" s="133"/>
+      <c r="T5" s="133"/>
       <c r="U5" s="13"/>
-      <c r="V5" s="103" t="s">
-        <v>32</v>
-      </c>
-      <c r="W5" s="104"/>
-      <c r="X5" s="104"/>
-      <c r="Y5" s="104"/>
-      <c r="Z5" s="104"/>
-      <c r="AA5" s="104"/>
-      <c r="AB5" s="104"/>
-      <c r="AC5" s="104"/>
-      <c r="AD5" s="104"/>
-      <c r="AE5" s="104"/>
-      <c r="AF5" s="105"/>
+      <c r="V5" s="134" t="s">
+        <v>31</v>
+      </c>
+      <c r="W5" s="135"/>
+      <c r="X5" s="135"/>
+      <c r="Y5" s="135"/>
+      <c r="Z5" s="135"/>
+      <c r="AA5" s="135"/>
+      <c r="AB5" s="135"/>
+      <c r="AC5" s="135"/>
+      <c r="AD5" s="135"/>
+      <c r="AE5" s="135"/>
+      <c r="AF5" s="136"/>
       <c r="AG5" s="58"/>
       <c r="AH5" s="58"/>
       <c r="AI5" s="58"/>
@@ -3862,7 +3852,7 @@
       <c r="AX5" s="16"/>
       <c r="AY5" s="17"/>
     </row>
-    <row r="6" spans="1:53" s="14" customFormat="1" ht="6.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:53" s="14" customFormat="1" ht="6.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.6">
       <c r="A6" s="23"/>
       <c r="B6" s="23"/>
       <c r="C6"/>
@@ -3900,47 +3890,47 @@
       <c r="AX6" s="16"/>
       <c r="AY6" s="17"/>
     </row>
-    <row r="7" spans="1:53" s="14" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A7" s="92" t="s">
+    <row r="7" spans="1:53" s="14" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.65">
+      <c r="A7" s="123" t="s">
         <v>19</v>
       </c>
-      <c r="B7" s="92"/>
-      <c r="C7" s="93"/>
-      <c r="D7" s="84" t="s">
+      <c r="B7" s="123"/>
+      <c r="C7" s="124"/>
+      <c r="D7" s="152" t="s">
         <v>25</v>
       </c>
-      <c r="E7" s="85"/>
-      <c r="F7" s="85"/>
-      <c r="G7" s="85"/>
-      <c r="H7" s="85"/>
-      <c r="I7" s="86"/>
-      <c r="J7" s="86"/>
-      <c r="K7" s="86"/>
-      <c r="L7" s="86"/>
-      <c r="M7" s="87"/>
+      <c r="E7" s="153"/>
+      <c r="F7" s="153"/>
+      <c r="G7" s="153"/>
+      <c r="H7" s="153"/>
+      <c r="I7" s="154"/>
+      <c r="J7" s="154"/>
+      <c r="K7" s="154"/>
+      <c r="L7" s="154"/>
+      <c r="M7" s="155"/>
       <c r="N7" s="54"/>
-      <c r="O7" s="102" t="s">
+      <c r="O7" s="133" t="s">
         <v>20</v>
       </c>
-      <c r="P7" s="102"/>
-      <c r="Q7" s="102"/>
-      <c r="R7" s="102"/>
-      <c r="S7" s="102"/>
-      <c r="T7" s="102"/>
+      <c r="P7" s="133"/>
+      <c r="Q7" s="133"/>
+      <c r="R7" s="133"/>
+      <c r="S7" s="133"/>
+      <c r="T7" s="133"/>
       <c r="U7" s="13"/>
-      <c r="V7" s="103" t="s">
+      <c r="V7" s="134" t="s">
         <v>26</v>
       </c>
-      <c r="W7" s="104"/>
-      <c r="X7" s="104"/>
-      <c r="Y7" s="104"/>
-      <c r="Z7" s="104"/>
-      <c r="AA7" s="104"/>
-      <c r="AB7" s="104"/>
-      <c r="AC7" s="104"/>
-      <c r="AD7" s="104"/>
-      <c r="AE7" s="104"/>
-      <c r="AF7" s="105"/>
+      <c r="W7" s="135"/>
+      <c r="X7" s="135"/>
+      <c r="Y7" s="135"/>
+      <c r="Z7" s="135"/>
+      <c r="AA7" s="135"/>
+      <c r="AB7" s="135"/>
+      <c r="AC7" s="135"/>
+      <c r="AD7" s="135"/>
+      <c r="AE7" s="135"/>
+      <c r="AF7" s="136"/>
       <c r="AG7" s="58"/>
       <c r="AH7" s="58"/>
       <c r="AI7" s="58"/>
@@ -3957,7 +3947,7 @@
       <c r="AX7" s="16"/>
       <c r="AY7" s="17"/>
     </row>
-    <row r="8" spans="1:53" s="14" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:53" s="14" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A8" s="21"/>
       <c r="B8" s="23"/>
       <c r="C8" s="54"/>
@@ -3994,9 +3984,9 @@
       <c r="AQ8" s="16"/>
       <c r="AR8" s="17"/>
     </row>
-    <row r="9" spans="1:53" s="14" customFormat="1" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A9" s="100"/>
-      <c r="B9" s="100"/>
+    <row r="9" spans="1:53" s="14" customFormat="1" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.6">
+      <c r="A9" s="131"/>
+      <c r="B9" s="131"/>
       <c r="C9" s="25"/>
       <c r="D9" s="54"/>
       <c r="E9" s="54"/>
@@ -4035,22 +4025,22 @@
       <c r="AQ9" s="16"/>
       <c r="AR9" s="17"/>
     </row>
-    <row r="10" spans="1:53" s="14" customFormat="1" ht="27" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A10" s="101" t="s">
+    <row r="10" spans="1:53" s="14" customFormat="1" ht="26" thickBot="1" x14ac:dyDescent="0.6">
+      <c r="A10" s="132" t="s">
         <v>2</v>
       </c>
-      <c r="B10" s="101"/>
-      <c r="C10" s="109">
+      <c r="B10" s="132"/>
+      <c r="C10" s="140">
         <v>45870</v>
       </c>
-      <c r="D10" s="110"/>
-      <c r="E10" s="111"/>
+      <c r="D10" s="141"/>
+      <c r="E10" s="142"/>
       <c r="G10" s="12"/>
       <c r="H10"/>
       <c r="I10" s="26"/>
-      <c r="J10" s="115"/>
-      <c r="K10" s="115"/>
-      <c r="L10" s="115"/>
+      <c r="J10" s="146"/>
+      <c r="K10" s="146"/>
+      <c r="L10" s="146"/>
       <c r="M10" s="27"/>
       <c r="N10" s="27"/>
       <c r="O10" s="27"/>
@@ -4074,7 +4064,7 @@
       <c r="AK10" s="10"/>
       <c r="AL10" s="10"/>
     </row>
-    <row r="11" spans="1:53" s="14" customFormat="1" ht="26.25" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:53" s="14" customFormat="1" ht="25.5" x14ac:dyDescent="0.55000000000000004">
       <c r="B11" s="23"/>
       <c r="H11" s="12"/>
       <c r="I11"/>
@@ -4100,7 +4090,7 @@
       <c r="AL11" s="10"/>
       <c r="AM11" s="10"/>
     </row>
-    <row r="12" spans="1:53" s="14" customFormat="1" ht="22.35" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:53" s="14" customFormat="1" ht="22.4" customHeight="1" thickBot="1" x14ac:dyDescent="0.6">
       <c r="A12" s="30"/>
       <c r="B12" s="30"/>
       <c r="C12" s="31"/>
@@ -4146,56 +4136,56 @@
       <c r="AT12" s="35"/>
       <c r="AU12" s="35"/>
     </row>
-    <row r="13" spans="1:53" s="37" customFormat="1" ht="33" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="94" t="s">
+    <row r="13" spans="1:53" s="37" customFormat="1" ht="33" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="125" t="s">
         <v>21</v>
       </c>
-      <c r="B13" s="95"/>
-      <c r="C13" s="112" t="s">
+      <c r="B13" s="126"/>
+      <c r="C13" s="143" t="s">
         <v>22</v>
       </c>
-      <c r="D13" s="106" t="s">
+      <c r="D13" s="137" t="s">
         <v>4</v>
       </c>
-      <c r="E13" s="107"/>
-      <c r="F13" s="107"/>
-      <c r="G13" s="107"/>
-      <c r="H13" s="107"/>
-      <c r="I13" s="107"/>
-      <c r="J13" s="107"/>
-      <c r="K13" s="107"/>
-      <c r="L13" s="107"/>
-      <c r="M13" s="107"/>
-      <c r="N13" s="107"/>
-      <c r="O13" s="107"/>
-      <c r="P13" s="107"/>
-      <c r="Q13" s="107"/>
-      <c r="R13" s="107"/>
-      <c r="S13" s="107"/>
-      <c r="T13" s="107"/>
-      <c r="U13" s="107"/>
-      <c r="V13" s="107"/>
-      <c r="W13" s="107"/>
-      <c r="X13" s="107"/>
-      <c r="Y13" s="107"/>
-      <c r="Z13" s="107"/>
-      <c r="AA13" s="107"/>
-      <c r="AB13" s="107"/>
-      <c r="AC13" s="107"/>
-      <c r="AD13" s="107"/>
-      <c r="AE13" s="107"/>
-      <c r="AF13" s="107"/>
-      <c r="AG13" s="107"/>
-      <c r="AH13" s="107"/>
-      <c r="AI13" s="107"/>
-      <c r="AJ13" s="108"/>
+      <c r="E13" s="138"/>
+      <c r="F13" s="138"/>
+      <c r="G13" s="138"/>
+      <c r="H13" s="138"/>
+      <c r="I13" s="138"/>
+      <c r="J13" s="138"/>
+      <c r="K13" s="138"/>
+      <c r="L13" s="138"/>
+      <c r="M13" s="138"/>
+      <c r="N13" s="138"/>
+      <c r="O13" s="138"/>
+      <c r="P13" s="138"/>
+      <c r="Q13" s="138"/>
+      <c r="R13" s="138"/>
+      <c r="S13" s="138"/>
+      <c r="T13" s="138"/>
+      <c r="U13" s="138"/>
+      <c r="V13" s="138"/>
+      <c r="W13" s="138"/>
+      <c r="X13" s="138"/>
+      <c r="Y13" s="138"/>
+      <c r="Z13" s="138"/>
+      <c r="AA13" s="138"/>
+      <c r="AB13" s="138"/>
+      <c r="AC13" s="138"/>
+      <c r="AD13" s="138"/>
+      <c r="AE13" s="138"/>
+      <c r="AF13" s="138"/>
+      <c r="AG13" s="138"/>
+      <c r="AH13" s="138"/>
+      <c r="AI13" s="138"/>
+      <c r="AJ13" s="139"/>
       <c r="AK13" s="36"/>
       <c r="AL13" s="36"/>
     </row>
-    <row r="14" spans="1:53" s="37" customFormat="1" ht="26.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="96"/>
-      <c r="B14" s="97"/>
-      <c r="C14" s="113"/>
+    <row r="14" spans="1:53" s="37" customFormat="1" ht="26.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A14" s="127"/>
+      <c r="B14" s="128"/>
+      <c r="C14" s="144"/>
       <c r="D14" s="59" t="str">
         <f t="shared" ref="D14:AG14" si="0">TEXT(D15, "ddd")</f>
         <v>Fri</v>
@@ -4319,10 +4309,10 @@
       <c r="AH14" s="60" t="s">
         <v>30</v>
       </c>
-      <c r="AI14" s="90" t="s">
+      <c r="AI14" s="121" t="s">
         <v>23</v>
       </c>
-      <c r="AJ14" s="116" t="s">
+      <c r="AJ14" s="147" t="s">
         <v>5</v>
       </c>
       <c r="AK14" s="36"/>
@@ -4343,10 +4333,10 @@
       <c r="AZ14" s="36"/>
       <c r="BA14" s="36"/>
     </row>
-    <row r="15" spans="1:53" s="38" customFormat="1" ht="26.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A15" s="98"/>
-      <c r="B15" s="99"/>
-      <c r="C15" s="114"/>
+    <row r="15" spans="1:53" s="38" customFormat="1" ht="26.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A15" s="129"/>
+      <c r="B15" s="130"/>
+      <c r="C15" s="145"/>
       <c r="D15" s="61">
         <f>C10</f>
         <v>45870</v>
@@ -4471,18 +4461,18 @@
         <f t="shared" si="4"/>
         <v>45900</v>
       </c>
-      <c r="AI15" s="91"/>
-      <c r="AJ15" s="117"/>
+      <c r="AI15" s="122"/>
+      <c r="AJ15" s="148"/>
       <c r="AR15" s="8"/>
       <c r="AS15" s="8"/>
       <c r="AT15" s="10"/>
       <c r="AU15" s="10"/>
     </row>
-    <row r="16" spans="1:53" s="39" customFormat="1" ht="26.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="88" t="s">
-        <v>33</v>
-      </c>
-      <c r="B16" s="89"/>
+    <row r="16" spans="1:53" s="39" customFormat="1" ht="26.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A16" s="156" t="s">
+        <v>32</v>
+      </c>
+      <c r="B16" s="157"/>
       <c r="C16" s="3" t="s">
         <v>27</v>
       </c>
@@ -4561,9 +4551,9 @@
       <c r="AT16" s="10"/>
       <c r="AU16" s="10"/>
     </row>
-    <row r="17" spans="1:47" s="39" customFormat="1" ht="26.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:47" s="39" customFormat="1" ht="26.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A17" s="82" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B17" s="83"/>
       <c r="C17" s="3" t="s">
@@ -4630,9 +4620,9 @@
       <c r="AT17" s="10"/>
       <c r="AU17" s="10"/>
     </row>
-    <row r="18" spans="1:47" s="39" customFormat="1" ht="26.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:47" s="39" customFormat="1" ht="26.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A18" s="82" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B18" s="83"/>
       <c r="C18" s="3" t="s">
@@ -4687,7 +4677,7 @@
       <c r="AT18" s="10"/>
       <c r="AU18" s="10"/>
     </row>
-    <row r="19" spans="1:47" s="39" customFormat="1" ht="26.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:47" s="39" customFormat="1" ht="26.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A19" s="82"/>
       <c r="B19" s="83"/>
       <c r="C19" s="3"/>
@@ -4709,19 +4699,19 @@
       <c r="S19" s="1"/>
       <c r="T19" s="1"/>
       <c r="U19" s="1"/>
-      <c r="V19" s="164"/>
-      <c r="W19" s="164"/>
-      <c r="X19" s="164"/>
-      <c r="Y19" s="164"/>
-      <c r="Z19" s="164"/>
-      <c r="AA19" s="164"/>
-      <c r="AB19" s="164"/>
-      <c r="AC19" s="164"/>
-      <c r="AD19" s="164"/>
-      <c r="AE19" s="164"/>
-      <c r="AF19" s="164"/>
-      <c r="AG19" s="164"/>
-      <c r="AH19" s="164"/>
+      <c r="V19" s="74"/>
+      <c r="W19" s="74"/>
+      <c r="X19" s="74"/>
+      <c r="Y19" s="74"/>
+      <c r="Z19" s="74"/>
+      <c r="AA19" s="74"/>
+      <c r="AB19" s="74"/>
+      <c r="AC19" s="74"/>
+      <c r="AD19" s="74"/>
+      <c r="AE19" s="74"/>
+      <c r="AF19" s="74"/>
+      <c r="AG19" s="74"/>
+      <c r="AH19" s="74"/>
       <c r="AI19" s="70"/>
       <c r="AJ19" s="63">
         <f t="shared" si="5"/>
@@ -4732,7 +4722,7 @@
       <c r="AT19" s="10"/>
       <c r="AU19" s="10"/>
     </row>
-    <row r="20" spans="1:47" s="39" customFormat="1" ht="26.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:47" s="39" customFormat="1" ht="26.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A20" s="82"/>
       <c r="B20" s="83"/>
       <c r="C20" s="3"/>
@@ -4754,19 +4744,19 @@
       <c r="S20" s="1"/>
       <c r="T20" s="1"/>
       <c r="U20" s="1"/>
-      <c r="V20" s="165"/>
-      <c r="W20" s="165"/>
-      <c r="X20" s="165"/>
-      <c r="Y20" s="165"/>
-      <c r="Z20" s="165"/>
-      <c r="AA20" s="165"/>
-      <c r="AB20" s="165"/>
-      <c r="AC20" s="165"/>
-      <c r="AD20" s="165"/>
-      <c r="AE20" s="165"/>
-      <c r="AF20" s="165"/>
-      <c r="AG20" s="165"/>
-      <c r="AH20" s="165"/>
+      <c r="V20" s="75"/>
+      <c r="W20" s="75"/>
+      <c r="X20" s="75"/>
+      <c r="Y20" s="75"/>
+      <c r="Z20" s="75"/>
+      <c r="AA20" s="75"/>
+      <c r="AB20" s="75"/>
+      <c r="AC20" s="75"/>
+      <c r="AD20" s="75"/>
+      <c r="AE20" s="75"/>
+      <c r="AF20" s="75"/>
+      <c r="AG20" s="75"/>
+      <c r="AH20" s="75"/>
       <c r="AI20" s="70"/>
       <c r="AJ20" s="63">
         <f t="shared" si="5"/>
@@ -4777,7 +4767,7 @@
       <c r="AT20" s="10"/>
       <c r="AU20" s="10"/>
     </row>
-    <row r="21" spans="1:47" s="39" customFormat="1" ht="26.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:47" s="39" customFormat="1" ht="26.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A21" s="82"/>
       <c r="B21" s="83"/>
       <c r="C21" s="3"/>
@@ -4822,7 +4812,7 @@
       <c r="AT21" s="10"/>
       <c r="AU21" s="10"/>
     </row>
-    <row r="22" spans="1:47" s="39" customFormat="1" ht="26.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:47" s="39" customFormat="1" ht="26.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A22" s="82"/>
       <c r="B22" s="83"/>
       <c r="C22" s="3"/>
@@ -4867,7 +4857,7 @@
       <c r="AT22" s="10"/>
       <c r="AU22" s="10"/>
     </row>
-    <row r="23" spans="1:47" s="39" customFormat="1" ht="26.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:47" s="39" customFormat="1" ht="26.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A23" s="82"/>
       <c r="B23" s="83"/>
       <c r="C23" s="3"/>
@@ -4912,7 +4902,7 @@
       <c r="AT23" s="10"/>
       <c r="AU23" s="10"/>
     </row>
-    <row r="24" spans="1:47" s="39" customFormat="1" ht="26.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:47" s="39" customFormat="1" ht="26.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A24" s="82"/>
       <c r="B24" s="83"/>
       <c r="C24" s="3"/>
@@ -4957,7 +4947,7 @@
       <c r="AT24" s="10"/>
       <c r="AU24" s="10"/>
     </row>
-    <row r="25" spans="1:47" s="39" customFormat="1" ht="26.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:47" s="39" customFormat="1" ht="26.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A25" s="82"/>
       <c r="B25" s="83"/>
       <c r="C25" s="3"/>
@@ -5002,7 +4992,7 @@
       <c r="AT25" s="10"/>
       <c r="AU25" s="10"/>
     </row>
-    <row r="26" spans="1:47" s="39" customFormat="1" ht="26.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:47" s="39" customFormat="1" ht="26.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A26" s="82"/>
       <c r="B26" s="83"/>
       <c r="C26" s="3"/>
@@ -5047,7 +5037,7 @@
       <c r="AT26" s="10"/>
       <c r="AU26" s="10"/>
     </row>
-    <row r="27" spans="1:47" s="39" customFormat="1" ht="26.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:47" s="39" customFormat="1" ht="26.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A27" s="82"/>
       <c r="B27" s="83"/>
       <c r="C27" s="3"/>
@@ -5092,7 +5082,7 @@
       <c r="AT27" s="10"/>
       <c r="AU27" s="10"/>
     </row>
-    <row r="28" spans="1:47" s="39" customFormat="1" ht="26.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:47" s="39" customFormat="1" ht="26.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A28" s="82"/>
       <c r="B28" s="83"/>
       <c r="C28" s="3"/>
@@ -5137,7 +5127,7 @@
       <c r="AT28" s="10"/>
       <c r="AU28" s="10"/>
     </row>
-    <row r="29" spans="1:47" s="39" customFormat="1" ht="26.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:47" s="39" customFormat="1" ht="26.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A29" s="82"/>
       <c r="B29" s="83"/>
       <c r="C29" s="3"/>
@@ -5182,7 +5172,7 @@
       <c r="AT29" s="10"/>
       <c r="AU29" s="10"/>
     </row>
-    <row r="30" spans="1:47" s="39" customFormat="1" ht="26.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:47" s="39" customFormat="1" ht="26.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A30" s="82"/>
       <c r="B30" s="83"/>
       <c r="C30" s="3"/>
@@ -5227,7 +5217,7 @@
       <c r="AT30" s="10"/>
       <c r="AU30" s="10"/>
     </row>
-    <row r="31" spans="1:47" s="39" customFormat="1" ht="26.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:47" s="39" customFormat="1" ht="26.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A31" s="82"/>
       <c r="B31" s="83"/>
       <c r="C31" s="3"/>
@@ -5272,7 +5262,7 @@
       <c r="AT31" s="10"/>
       <c r="AU31" s="10"/>
     </row>
-    <row r="32" spans="1:47" s="40" customFormat="1" ht="26.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:47" s="40" customFormat="1" ht="26.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A32" s="82"/>
       <c r="B32" s="83"/>
       <c r="C32" s="3"/>
@@ -5317,7 +5307,7 @@
       <c r="AT32" s="10"/>
       <c r="AU32" s="10"/>
     </row>
-    <row r="33" spans="1:47" s="40" customFormat="1" ht="26.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:47" s="40" customFormat="1" ht="26.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A33" s="82"/>
       <c r="B33" s="83"/>
       <c r="C33" s="3"/>
@@ -5362,7 +5352,7 @@
       <c r="AT33" s="10"/>
       <c r="AU33" s="10"/>
     </row>
-    <row r="34" spans="1:47" s="40" customFormat="1" ht="26.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:47" s="40" customFormat="1" ht="26.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A34" s="82"/>
       <c r="B34" s="83"/>
       <c r="C34" s="3"/>
@@ -5407,9 +5397,9 @@
       <c r="AT34" s="41"/>
       <c r="AU34" s="10"/>
     </row>
-    <row r="35" spans="1:47" s="40" customFormat="1" ht="26.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="140"/>
-      <c r="B35" s="141"/>
+    <row r="35" spans="1:47" s="40" customFormat="1" ht="26.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A35" s="80"/>
+      <c r="B35" s="81"/>
       <c r="C35" s="4"/>
       <c r="D35" s="2"/>
       <c r="E35" s="2"/>
@@ -5452,12 +5442,12 @@
       <c r="AT35" s="10"/>
       <c r="AU35" s="10"/>
     </row>
-    <row r="36" spans="1:47" s="38" customFormat="1" ht="27" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A36" s="137" t="s">
+    <row r="36" spans="1:47" s="38" customFormat="1" ht="27" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A36" s="77" t="s">
         <v>6</v>
       </c>
-      <c r="B36" s="138"/>
-      <c r="C36" s="139"/>
+      <c r="B36" s="78"/>
+      <c r="C36" s="79"/>
       <c r="D36" s="65">
         <f t="shared" ref="D36:AJ36" si="6">SUM(D16:D35)</f>
         <v>1</v>
@@ -5531,55 +5521,55 @@
         <v>1</v>
       </c>
       <c r="V36" s="65">
-        <f>SUM(V16:V35)</f>
+        <f t="shared" ref="V36:AH36" si="7">SUM(V16:V35)</f>
         <v>1</v>
       </c>
       <c r="W36" s="65">
-        <f>SUM(W16:W35)</f>
+        <f t="shared" si="7"/>
         <v>1</v>
       </c>
       <c r="X36" s="65">
-        <f>SUM(X16:X35)</f>
+        <f t="shared" si="7"/>
         <v>1</v>
       </c>
       <c r="Y36" s="65">
-        <f>SUM(Y16:Y35)</f>
+        <f t="shared" si="7"/>
         <v>1</v>
       </c>
       <c r="Z36" s="65">
-        <f>SUM(Z16:Z35)</f>
+        <f t="shared" si="7"/>
         <v>1</v>
       </c>
       <c r="AA36" s="65">
-        <f>SUM(AA16:AA35)</f>
+        <f t="shared" si="7"/>
         <v>1</v>
       </c>
       <c r="AB36" s="65">
-        <f>SUM(AB16:AB35)</f>
+        <f t="shared" si="7"/>
         <v>1</v>
       </c>
       <c r="AC36" s="65">
-        <f>SUM(AC16:AC35)</f>
+        <f t="shared" si="7"/>
         <v>1</v>
       </c>
       <c r="AD36" s="65">
-        <f>SUM(AD16:AD35)</f>
+        <f t="shared" si="7"/>
         <v>1</v>
       </c>
       <c r="AE36" s="65">
-        <f>SUM(AE16:AE35)</f>
+        <f t="shared" si="7"/>
         <v>1</v>
       </c>
       <c r="AF36" s="65">
-        <f>SUM(AF16:AF35)</f>
+        <f t="shared" si="7"/>
         <v>1</v>
       </c>
       <c r="AG36" s="65">
-        <f>SUM(AG16:AG35)</f>
+        <f t="shared" si="7"/>
         <v>1</v>
       </c>
       <c r="AH36" s="65">
-        <f>SUM(AH16:AH35)</f>
+        <f t="shared" si="7"/>
         <v>1</v>
       </c>
       <c r="AI36" s="65">
@@ -5595,7 +5585,7 @@
       <c r="AT36" s="10"/>
       <c r="AU36" s="10"/>
     </row>
-    <row r="37" spans="1:47" ht="8.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:47" ht="8.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A37" s="42"/>
       <c r="B37" s="43"/>
       <c r="C37" s="43"/>
@@ -5637,193 +5627,193 @@
       <c r="AT37" s="10"/>
       <c r="AU37" s="10"/>
     </row>
-    <row r="38" spans="1:47" ht="36.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A38" s="129" t="s">
+    <row r="38" spans="1:47" ht="36.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A38" s="114" t="s">
         <v>7</v>
       </c>
-      <c r="B38" s="130"/>
-      <c r="C38" s="130"/>
-      <c r="D38" s="131"/>
-      <c r="E38" s="132"/>
-      <c r="F38" s="132"/>
-      <c r="G38" s="132"/>
-      <c r="H38" s="132"/>
-      <c r="I38" s="133"/>
-      <c r="J38" s="134" t="s">
+      <c r="B38" s="115"/>
+      <c r="C38" s="115"/>
+      <c r="D38" s="116"/>
+      <c r="E38" s="117"/>
+      <c r="F38" s="117"/>
+      <c r="G38" s="117"/>
+      <c r="H38" s="117"/>
+      <c r="I38" s="118"/>
+      <c r="J38" s="119" t="s">
         <v>16</v>
       </c>
-      <c r="K38" s="134"/>
-      <c r="L38" s="134"/>
-      <c r="M38" s="134"/>
-      <c r="N38" s="135"/>
-      <c r="O38" s="124"/>
-      <c r="P38" s="125"/>
-      <c r="Q38" s="125"/>
-      <c r="R38" s="125"/>
-      <c r="S38" s="125"/>
-      <c r="T38" s="125"/>
-      <c r="U38" s="125"/>
-      <c r="V38" s="125"/>
-      <c r="W38" s="126" t="s">
+      <c r="K38" s="119"/>
+      <c r="L38" s="119"/>
+      <c r="M38" s="119"/>
+      <c r="N38" s="120"/>
+      <c r="O38" s="109"/>
+      <c r="P38" s="110"/>
+      <c r="Q38" s="110"/>
+      <c r="R38" s="110"/>
+      <c r="S38" s="110"/>
+      <c r="T38" s="110"/>
+      <c r="U38" s="110"/>
+      <c r="V38" s="110"/>
+      <c r="W38" s="111" t="s">
         <v>8</v>
       </c>
-      <c r="X38" s="127"/>
-      <c r="Y38" s="127"/>
-      <c r="Z38" s="127"/>
-      <c r="AA38" s="127"/>
-      <c r="AB38" s="127"/>
-      <c r="AC38" s="127"/>
-      <c r="AD38" s="127"/>
-      <c r="AE38" s="127"/>
-      <c r="AF38" s="127"/>
-      <c r="AG38" s="127"/>
-      <c r="AH38" s="127"/>
-      <c r="AI38" s="127"/>
-      <c r="AJ38" s="128"/>
+      <c r="X38" s="112"/>
+      <c r="Y38" s="112"/>
+      <c r="Z38" s="112"/>
+      <c r="AA38" s="112"/>
+      <c r="AB38" s="112"/>
+      <c r="AC38" s="112"/>
+      <c r="AD38" s="112"/>
+      <c r="AE38" s="112"/>
+      <c r="AF38" s="112"/>
+      <c r="AG38" s="112"/>
+      <c r="AH38" s="112"/>
+      <c r="AI38" s="112"/>
+      <c r="AJ38" s="113"/>
       <c r="AQ38" s="8"/>
       <c r="AR38" s="8"/>
       <c r="AS38" s="10"/>
       <c r="AT38" s="10"/>
     </row>
-    <row r="39" spans="1:47" ht="36.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A39" s="74" t="s">
+    <row r="39" spans="1:47" ht="36.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A39" s="158" t="s">
         <v>9</v>
       </c>
-      <c r="B39" s="75"/>
-      <c r="C39" s="75"/>
-      <c r="D39" s="79"/>
-      <c r="E39" s="80"/>
-      <c r="F39" s="80"/>
-      <c r="G39" s="80"/>
-      <c r="H39" s="80"/>
-      <c r="I39" s="81"/>
-      <c r="J39" s="156" t="s">
+      <c r="B39" s="159"/>
+      <c r="C39" s="159"/>
+      <c r="D39" s="163"/>
+      <c r="E39" s="164"/>
+      <c r="F39" s="164"/>
+      <c r="G39" s="164"/>
+      <c r="H39" s="164"/>
+      <c r="I39" s="165"/>
+      <c r="J39" s="101" t="s">
         <v>9</v>
       </c>
-      <c r="K39" s="157"/>
-      <c r="L39" s="157"/>
-      <c r="M39" s="157"/>
-      <c r="N39" s="158"/>
-      <c r="O39" s="162"/>
-      <c r="P39" s="163"/>
-      <c r="Q39" s="163"/>
-      <c r="R39" s="163"/>
-      <c r="S39" s="163"/>
-      <c r="T39" s="163"/>
-      <c r="U39" s="163"/>
-      <c r="V39" s="163"/>
-      <c r="W39" s="121"/>
-      <c r="X39" s="122"/>
-      <c r="Y39" s="122"/>
-      <c r="Z39" s="122"/>
-      <c r="AA39" s="122"/>
-      <c r="AB39" s="122"/>
-      <c r="AC39" s="122"/>
-      <c r="AD39" s="122"/>
-      <c r="AE39" s="122"/>
-      <c r="AF39" s="122"/>
-      <c r="AG39" s="122"/>
-      <c r="AH39" s="122"/>
-      <c r="AI39" s="122"/>
-      <c r="AJ39" s="123"/>
+      <c r="K39" s="102"/>
+      <c r="L39" s="102"/>
+      <c r="M39" s="102"/>
+      <c r="N39" s="103"/>
+      <c r="O39" s="107"/>
+      <c r="P39" s="108"/>
+      <c r="Q39" s="108"/>
+      <c r="R39" s="108"/>
+      <c r="S39" s="108"/>
+      <c r="T39" s="108"/>
+      <c r="U39" s="108"/>
+      <c r="V39" s="108"/>
+      <c r="W39" s="84"/>
+      <c r="X39" s="85"/>
+      <c r="Y39" s="85"/>
+      <c r="Z39" s="85"/>
+      <c r="AA39" s="85"/>
+      <c r="AB39" s="85"/>
+      <c r="AC39" s="85"/>
+      <c r="AD39" s="85"/>
+      <c r="AE39" s="85"/>
+      <c r="AF39" s="85"/>
+      <c r="AG39" s="85"/>
+      <c r="AH39" s="85"/>
+      <c r="AI39" s="85"/>
+      <c r="AJ39" s="86"/>
       <c r="AQ39" s="8"/>
       <c r="AR39" s="8"/>
       <c r="AS39" s="10"/>
       <c r="AT39" s="10"/>
     </row>
-    <row r="40" spans="1:47" ht="36.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A40" s="74" t="s">
+    <row r="40" spans="1:47" ht="36.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A40" s="158" t="s">
         <v>10</v>
       </c>
-      <c r="B40" s="75"/>
-      <c r="C40" s="75"/>
-      <c r="D40" s="76"/>
-      <c r="E40" s="77"/>
-      <c r="F40" s="77"/>
-      <c r="G40" s="77"/>
-      <c r="H40" s="77"/>
-      <c r="I40" s="78"/>
-      <c r="J40" s="156" t="s">
+      <c r="B40" s="159"/>
+      <c r="C40" s="159"/>
+      <c r="D40" s="160"/>
+      <c r="E40" s="161"/>
+      <c r="F40" s="161"/>
+      <c r="G40" s="161"/>
+      <c r="H40" s="161"/>
+      <c r="I40" s="162"/>
+      <c r="J40" s="101" t="s">
         <v>10</v>
       </c>
-      <c r="K40" s="157"/>
-      <c r="L40" s="157"/>
-      <c r="M40" s="157"/>
-      <c r="N40" s="158"/>
-      <c r="O40" s="159"/>
-      <c r="P40" s="160"/>
-      <c r="Q40" s="160"/>
-      <c r="R40" s="160"/>
-      <c r="S40" s="160"/>
-      <c r="T40" s="160"/>
-      <c r="U40" s="160"/>
-      <c r="V40" s="161"/>
-      <c r="W40" s="121"/>
-      <c r="X40" s="122"/>
-      <c r="Y40" s="122"/>
-      <c r="Z40" s="122"/>
-      <c r="AA40" s="122"/>
-      <c r="AB40" s="122"/>
-      <c r="AC40" s="122"/>
-      <c r="AD40" s="122"/>
-      <c r="AE40" s="122"/>
-      <c r="AF40" s="122"/>
-      <c r="AG40" s="122"/>
-      <c r="AH40" s="122"/>
-      <c r="AI40" s="122"/>
-      <c r="AJ40" s="123"/>
+      <c r="K40" s="102"/>
+      <c r="L40" s="102"/>
+      <c r="M40" s="102"/>
+      <c r="N40" s="103"/>
+      <c r="O40" s="104"/>
+      <c r="P40" s="105"/>
+      <c r="Q40" s="105"/>
+      <c r="R40" s="105"/>
+      <c r="S40" s="105"/>
+      <c r="T40" s="105"/>
+      <c r="U40" s="105"/>
+      <c r="V40" s="106"/>
+      <c r="W40" s="84"/>
+      <c r="X40" s="85"/>
+      <c r="Y40" s="85"/>
+      <c r="Z40" s="85"/>
+      <c r="AA40" s="85"/>
+      <c r="AB40" s="85"/>
+      <c r="AC40" s="85"/>
+      <c r="AD40" s="85"/>
+      <c r="AE40" s="85"/>
+      <c r="AF40" s="85"/>
+      <c r="AG40" s="85"/>
+      <c r="AH40" s="85"/>
+      <c r="AI40" s="85"/>
+      <c r="AJ40" s="86"/>
       <c r="AQ40" s="8"/>
       <c r="AR40" s="8"/>
       <c r="AS40" s="10"/>
       <c r="AT40" s="10"/>
     </row>
-    <row r="41" spans="1:47" ht="36.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A41" s="145" t="s">
+    <row r="41" spans="1:47" ht="36.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A41" s="90" t="s">
         <v>11</v>
       </c>
-      <c r="B41" s="146"/>
-      <c r="C41" s="146"/>
-      <c r="D41" s="147"/>
-      <c r="E41" s="148"/>
-      <c r="F41" s="148"/>
-      <c r="G41" s="148"/>
-      <c r="H41" s="148"/>
-      <c r="I41" s="149"/>
-      <c r="J41" s="153" t="s">
+      <c r="B41" s="91"/>
+      <c r="C41" s="91"/>
+      <c r="D41" s="92"/>
+      <c r="E41" s="93"/>
+      <c r="F41" s="93"/>
+      <c r="G41" s="93"/>
+      <c r="H41" s="93"/>
+      <c r="I41" s="94"/>
+      <c r="J41" s="98" t="s">
         <v>11</v>
       </c>
-      <c r="K41" s="154"/>
-      <c r="L41" s="154"/>
-      <c r="M41" s="154"/>
-      <c r="N41" s="155"/>
-      <c r="O41" s="150"/>
-      <c r="P41" s="151"/>
-      <c r="Q41" s="151"/>
-      <c r="R41" s="151"/>
-      <c r="S41" s="151"/>
-      <c r="T41" s="151"/>
-      <c r="U41" s="151"/>
-      <c r="V41" s="152"/>
-      <c r="W41" s="142"/>
-      <c r="X41" s="143"/>
-      <c r="Y41" s="143"/>
-      <c r="Z41" s="143"/>
-      <c r="AA41" s="143"/>
-      <c r="AB41" s="143"/>
-      <c r="AC41" s="143"/>
-      <c r="AD41" s="143"/>
-      <c r="AE41" s="143"/>
-      <c r="AF41" s="143"/>
-      <c r="AG41" s="143"/>
-      <c r="AH41" s="143"/>
-      <c r="AI41" s="143"/>
-      <c r="AJ41" s="144"/>
+      <c r="K41" s="99"/>
+      <c r="L41" s="99"/>
+      <c r="M41" s="99"/>
+      <c r="N41" s="100"/>
+      <c r="O41" s="95"/>
+      <c r="P41" s="96"/>
+      <c r="Q41" s="96"/>
+      <c r="R41" s="96"/>
+      <c r="S41" s="96"/>
+      <c r="T41" s="96"/>
+      <c r="U41" s="96"/>
+      <c r="V41" s="97"/>
+      <c r="W41" s="87"/>
+      <c r="X41" s="88"/>
+      <c r="Y41" s="88"/>
+      <c r="Z41" s="88"/>
+      <c r="AA41" s="88"/>
+      <c r="AB41" s="88"/>
+      <c r="AC41" s="88"/>
+      <c r="AD41" s="88"/>
+      <c r="AE41" s="88"/>
+      <c r="AF41" s="88"/>
+      <c r="AG41" s="88"/>
+      <c r="AH41" s="88"/>
+      <c r="AI41" s="88"/>
+      <c r="AJ41" s="89"/>
       <c r="AQ41" s="8"/>
       <c r="AR41" s="8"/>
       <c r="AS41" s="10"/>
       <c r="AT41" s="10"/>
     </row>
-    <row r="42" spans="1:47" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:47" ht="16" x14ac:dyDescent="0.35">
       <c r="A42" s="12"/>
       <c r="B42" s="12"/>
       <c r="C42" s="12"/>
@@ -5864,91 +5854,91 @@
       <c r="AS42" s="10"/>
       <c r="AT42" s="10"/>
     </row>
-    <row r="43" spans="1:47" ht="30.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A43" s="136" t="s">
+    <row r="43" spans="1:47" ht="30.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A43" s="76" t="s">
         <v>12</v>
       </c>
-      <c r="B43" s="136"/>
-      <c r="C43" s="136"/>
-      <c r="D43" s="136"/>
-      <c r="E43" s="136"/>
-      <c r="F43" s="136"/>
-      <c r="G43" s="136"/>
-      <c r="H43" s="136"/>
-      <c r="I43" s="136"/>
-      <c r="J43" s="136"/>
-      <c r="K43" s="136"/>
-      <c r="L43" s="136"/>
-      <c r="M43" s="136"/>
-      <c r="N43" s="136"/>
-      <c r="O43" s="136"/>
-      <c r="P43" s="136"/>
-      <c r="Q43" s="136"/>
-      <c r="R43" s="136"/>
-      <c r="S43" s="136"/>
-      <c r="T43" s="136"/>
-      <c r="U43" s="136"/>
-      <c r="V43" s="136"/>
-      <c r="W43" s="136"/>
-      <c r="X43" s="136"/>
-      <c r="Y43" s="136"/>
-      <c r="Z43" s="136"/>
-      <c r="AA43" s="136"/>
-      <c r="AB43" s="136"/>
-      <c r="AC43" s="136"/>
-      <c r="AD43" s="136"/>
-      <c r="AE43" s="136"/>
-      <c r="AF43" s="136"/>
-      <c r="AG43" s="136"/>
-      <c r="AH43" s="136"/>
-      <c r="AI43" s="136"/>
-      <c r="AJ43" s="136"/>
+      <c r="B43" s="76"/>
+      <c r="C43" s="76"/>
+      <c r="D43" s="76"/>
+      <c r="E43" s="76"/>
+      <c r="F43" s="76"/>
+      <c r="G43" s="76"/>
+      <c r="H43" s="76"/>
+      <c r="I43" s="76"/>
+      <c r="J43" s="76"/>
+      <c r="K43" s="76"/>
+      <c r="L43" s="76"/>
+      <c r="M43" s="76"/>
+      <c r="N43" s="76"/>
+      <c r="O43" s="76"/>
+      <c r="P43" s="76"/>
+      <c r="Q43" s="76"/>
+      <c r="R43" s="76"/>
+      <c r="S43" s="76"/>
+      <c r="T43" s="76"/>
+      <c r="U43" s="76"/>
+      <c r="V43" s="76"/>
+      <c r="W43" s="76"/>
+      <c r="X43" s="76"/>
+      <c r="Y43" s="76"/>
+      <c r="Z43" s="76"/>
+      <c r="AA43" s="76"/>
+      <c r="AB43" s="76"/>
+      <c r="AC43" s="76"/>
+      <c r="AD43" s="76"/>
+      <c r="AE43" s="76"/>
+      <c r="AF43" s="76"/>
+      <c r="AG43" s="76"/>
+      <c r="AH43" s="76"/>
+      <c r="AI43" s="76"/>
+      <c r="AJ43" s="76"/>
       <c r="AK43" s="45"/>
       <c r="AL43" s="45"/>
     </row>
-    <row r="44" spans="1:47" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A44" s="136" t="s">
+    <row r="44" spans="1:47" ht="35.25" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A44" s="76" t="s">
         <v>13</v>
       </c>
-      <c r="B44" s="136"/>
-      <c r="C44" s="136"/>
-      <c r="D44" s="136"/>
-      <c r="E44" s="136"/>
-      <c r="F44" s="136"/>
-      <c r="G44" s="136"/>
-      <c r="H44" s="136"/>
-      <c r="I44" s="136"/>
-      <c r="J44" s="136"/>
-      <c r="K44" s="136"/>
-      <c r="L44" s="136"/>
-      <c r="M44" s="136"/>
-      <c r="N44" s="136"/>
-      <c r="O44" s="136"/>
-      <c r="P44" s="136"/>
-      <c r="Q44" s="136"/>
-      <c r="R44" s="136"/>
-      <c r="S44" s="136"/>
-      <c r="T44" s="136"/>
-      <c r="U44" s="136"/>
-      <c r="V44" s="136"/>
-      <c r="W44" s="136"/>
-      <c r="X44" s="136"/>
-      <c r="Y44" s="136"/>
-      <c r="Z44" s="136"/>
-      <c r="AA44" s="136"/>
-      <c r="AB44" s="136"/>
-      <c r="AC44" s="136"/>
-      <c r="AD44" s="136"/>
-      <c r="AE44" s="136"/>
-      <c r="AF44" s="136"/>
-      <c r="AG44" s="136"/>
-      <c r="AH44" s="136"/>
-      <c r="AI44" s="136"/>
-      <c r="AJ44" s="136"/>
+      <c r="B44" s="76"/>
+      <c r="C44" s="76"/>
+      <c r="D44" s="76"/>
+      <c r="E44" s="76"/>
+      <c r="F44" s="76"/>
+      <c r="G44" s="76"/>
+      <c r="H44" s="76"/>
+      <c r="I44" s="76"/>
+      <c r="J44" s="76"/>
+      <c r="K44" s="76"/>
+      <c r="L44" s="76"/>
+      <c r="M44" s="76"/>
+      <c r="N44" s="76"/>
+      <c r="O44" s="76"/>
+      <c r="P44" s="76"/>
+      <c r="Q44" s="76"/>
+      <c r="R44" s="76"/>
+      <c r="S44" s="76"/>
+      <c r="T44" s="76"/>
+      <c r="U44" s="76"/>
+      <c r="V44" s="76"/>
+      <c r="W44" s="76"/>
+      <c r="X44" s="76"/>
+      <c r="Y44" s="76"/>
+      <c r="Z44" s="76"/>
+      <c r="AA44" s="76"/>
+      <c r="AB44" s="76"/>
+      <c r="AC44" s="76"/>
+      <c r="AD44" s="76"/>
+      <c r="AE44" s="76"/>
+      <c r="AF44" s="76"/>
+      <c r="AG44" s="76"/>
+      <c r="AH44" s="76"/>
+      <c r="AI44" s="76"/>
+      <c r="AJ44" s="76"/>
       <c r="AK44" s="45"/>
       <c r="AL44" s="45"/>
     </row>
-    <row r="45" spans="1:47" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:47" ht="18" x14ac:dyDescent="0.4">
       <c r="A45" s="46"/>
       <c r="B45" s="47"/>
       <c r="C45" s="46"/>
@@ -5988,7 +5978,7 @@
       <c r="AK45" s="45"/>
       <c r="AL45" s="45"/>
     </row>
-    <row r="46" spans="1:47" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:47" ht="18" x14ac:dyDescent="0.4">
       <c r="A46" s="46"/>
       <c r="B46" s="47"/>
       <c r="C46" s="46"/>
@@ -6028,185 +6018,229 @@
       <c r="AK46" s="45"/>
       <c r="AL46" s="45"/>
     </row>
-    <row r="51" spans="4:7" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="51" spans="4:7" ht="16" x14ac:dyDescent="0.35">
       <c r="D51" s="48"/>
     </row>
-    <row r="52" spans="4:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="52" spans="4:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D52" s="49"/>
       <c r="E52" s="49"/>
       <c r="F52" s="50"/>
       <c r="G52" s="50"/>
     </row>
-    <row r="53" spans="4:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="53" spans="4:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="D53" s="51"/>
       <c r="E53" s="48"/>
       <c r="F53" s="52"/>
       <c r="G53" s="52"/>
     </row>
-    <row r="54" spans="4:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="54" spans="4:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="D54" s="51"/>
       <c r="E54" s="48"/>
       <c r="F54" s="52"/>
       <c r="G54" s="52"/>
     </row>
-    <row r="55" spans="4:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="55" spans="4:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="D55" s="51"/>
       <c r="E55" s="48"/>
       <c r="F55" s="52"/>
       <c r="G55" s="52"/>
     </row>
-    <row r="56" spans="4:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="56" spans="4:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="D56" s="51"/>
       <c r="E56" s="48"/>
       <c r="F56" s="52"/>
       <c r="G56" s="52"/>
     </row>
-    <row r="57" spans="4:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="57" spans="4:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="D57" s="51"/>
       <c r="E57" s="48"/>
       <c r="F57" s="52"/>
       <c r="G57" s="52"/>
     </row>
-    <row r="58" spans="4:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="58" spans="4:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="D58" s="51"/>
       <c r="E58" s="48"/>
       <c r="F58" s="52"/>
       <c r="G58" s="52"/>
     </row>
-    <row r="59" spans="4:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="59" spans="4:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="D59" s="51"/>
       <c r="E59" s="48"/>
       <c r="F59" s="52"/>
       <c r="G59" s="52"/>
     </row>
-    <row r="60" spans="4:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="60" spans="4:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="D60" s="51"/>
       <c r="E60" s="48"/>
       <c r="F60" s="52"/>
       <c r="G60" s="52"/>
     </row>
-    <row r="61" spans="4:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="61" spans="4:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="D61" s="51"/>
       <c r="E61" s="48"/>
       <c r="F61" s="52"/>
       <c r="G61" s="52"/>
     </row>
-    <row r="62" spans="4:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="62" spans="4:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="D62" s="51"/>
       <c r="E62" s="48"/>
       <c r="F62" s="52"/>
       <c r="G62" s="52"/>
     </row>
-    <row r="63" spans="4:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="63" spans="4:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="D63" s="51"/>
       <c r="E63" s="48"/>
       <c r="F63" s="52"/>
       <c r="G63" s="52"/>
     </row>
-    <row r="64" spans="4:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="64" spans="4:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="D64" s="51"/>
       <c r="E64" s="48"/>
       <c r="F64" s="52"/>
       <c r="G64" s="52"/>
     </row>
-    <row r="65" spans="4:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="65" spans="4:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="D65" s="6"/>
       <c r="E65" s="48"/>
       <c r="F65" s="52"/>
       <c r="G65" s="52"/>
     </row>
-    <row r="66" spans="4:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="66" spans="4:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="E66" s="48"/>
       <c r="F66" s="52"/>
       <c r="G66" s="52"/>
     </row>
-    <row r="67" spans="4:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="67" spans="4:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="E67" s="48"/>
       <c r="F67" s="52"/>
       <c r="G67" s="52"/>
     </row>
-    <row r="68" spans="4:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="68" spans="4:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="E68" s="48"/>
       <c r="F68" s="52"/>
       <c r="G68" s="52"/>
     </row>
-    <row r="69" spans="4:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="69" spans="4:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="E69" s="48"/>
       <c r="F69" s="52"/>
       <c r="G69" s="52"/>
     </row>
-    <row r="70" spans="4:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="70" spans="4:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="E70" s="48"/>
       <c r="F70" s="53"/>
       <c r="G70" s="52"/>
     </row>
-    <row r="71" spans="4:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="71" spans="4:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="E71" s="48"/>
       <c r="F71" s="52"/>
       <c r="G71" s="52"/>
     </row>
-    <row r="72" spans="4:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="72" spans="4:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="E72" s="48"/>
       <c r="F72" s="52"/>
       <c r="G72" s="52"/>
     </row>
-    <row r="73" spans="4:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="73" spans="4:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="E73" s="48"/>
       <c r="F73" s="52"/>
       <c r="G73" s="52"/>
     </row>
-    <row r="74" spans="4:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="74" spans="4:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="E74" s="48"/>
       <c r="F74" s="52"/>
       <c r="G74" s="52"/>
     </row>
-    <row r="75" spans="4:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="75" spans="4:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="E75" s="48"/>
       <c r="F75" s="52"/>
       <c r="G75" s="52"/>
     </row>
-    <row r="76" spans="4:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="76" spans="4:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="E76" s="48"/>
       <c r="F76" s="52"/>
       <c r="G76" s="52"/>
     </row>
-    <row r="77" spans="4:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="77" spans="4:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="E77" s="48"/>
       <c r="F77" s="52"/>
       <c r="G77" s="52"/>
     </row>
-    <row r="78" spans="4:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="78" spans="4:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="E78" s="48"/>
       <c r="F78" s="52"/>
       <c r="G78" s="52"/>
     </row>
-    <row r="79" spans="4:7" ht="13.5" x14ac:dyDescent="0.25">
+    <row r="79" spans="4:7" x14ac:dyDescent="0.3">
       <c r="E79" s="6"/>
       <c r="F79" s="6"/>
       <c r="G79" s="6"/>
     </row>
-    <row r="80" spans="4:7" ht="13.5" x14ac:dyDescent="0.25">
+    <row r="80" spans="4:7" x14ac:dyDescent="0.3">
       <c r="E80" s="6"/>
       <c r="F80" s="6"/>
       <c r="G80" s="6"/>
     </row>
-    <row r="81" spans="5:7" ht="13.5" x14ac:dyDescent="0.25">
+    <row r="81" spans="5:7" x14ac:dyDescent="0.3">
       <c r="E81" s="6"/>
       <c r="F81" s="6"/>
       <c r="G81" s="6"/>
     </row>
-    <row r="82" spans="5:7" ht="13.5" x14ac:dyDescent="0.25">
+    <row r="82" spans="5:7" x14ac:dyDescent="0.3">
       <c r="E82" s="6"/>
       <c r="F82" s="6"/>
       <c r="G82" s="6"/>
     </row>
-    <row r="83" spans="5:7" ht="13.5" x14ac:dyDescent="0.25">
+    <row r="83" spans="5:7" x14ac:dyDescent="0.3">
       <c r="E83" s="6"/>
       <c r="F83" s="6"/>
       <c r="G83" s="6"/>
     </row>
   </sheetData>
   <mergeCells count="60">
+    <mergeCell ref="A40:C40"/>
+    <mergeCell ref="D40:I40"/>
+    <mergeCell ref="D39:I39"/>
+    <mergeCell ref="A24:B24"/>
+    <mergeCell ref="A30:B30"/>
+    <mergeCell ref="A25:B25"/>
+    <mergeCell ref="A26:B26"/>
+    <mergeCell ref="A27:B27"/>
+    <mergeCell ref="A28:B28"/>
+    <mergeCell ref="A29:B29"/>
+    <mergeCell ref="A31:B31"/>
+    <mergeCell ref="A32:B32"/>
+    <mergeCell ref="A39:C39"/>
+    <mergeCell ref="A23:B23"/>
+    <mergeCell ref="A17:B17"/>
+    <mergeCell ref="A18:B18"/>
+    <mergeCell ref="D7:M7"/>
+    <mergeCell ref="A19:B19"/>
+    <mergeCell ref="A20:B20"/>
+    <mergeCell ref="A21:B21"/>
+    <mergeCell ref="A22:B22"/>
+    <mergeCell ref="A16:B16"/>
+    <mergeCell ref="AI14:AI15"/>
+    <mergeCell ref="A5:C5"/>
+    <mergeCell ref="A13:B15"/>
+    <mergeCell ref="A9:B9"/>
+    <mergeCell ref="A10:B10"/>
+    <mergeCell ref="O7:T7"/>
+    <mergeCell ref="V5:AF5"/>
+    <mergeCell ref="V7:AF7"/>
+    <mergeCell ref="D13:AJ13"/>
+    <mergeCell ref="C10:E10"/>
+    <mergeCell ref="C13:C15"/>
+    <mergeCell ref="A7:C7"/>
+    <mergeCell ref="J10:L10"/>
+    <mergeCell ref="AJ14:AJ15"/>
+    <mergeCell ref="Q5:T5"/>
+    <mergeCell ref="D5:M5"/>
+    <mergeCell ref="W39:AJ39"/>
+    <mergeCell ref="O38:V38"/>
+    <mergeCell ref="W38:AJ38"/>
+    <mergeCell ref="A38:C38"/>
+    <mergeCell ref="D38:I38"/>
+    <mergeCell ref="J38:N38"/>
     <mergeCell ref="A43:AJ43"/>
     <mergeCell ref="A44:AJ44"/>
     <mergeCell ref="A36:C36"/>
@@ -6223,50 +6257,6 @@
     <mergeCell ref="J40:N40"/>
     <mergeCell ref="O40:V40"/>
     <mergeCell ref="O39:V39"/>
-    <mergeCell ref="W39:AJ39"/>
-    <mergeCell ref="O38:V38"/>
-    <mergeCell ref="W38:AJ38"/>
-    <mergeCell ref="A38:C38"/>
-    <mergeCell ref="D38:I38"/>
-    <mergeCell ref="J38:N38"/>
-    <mergeCell ref="AI14:AI15"/>
-    <mergeCell ref="A5:C5"/>
-    <mergeCell ref="A13:B15"/>
-    <mergeCell ref="A9:B9"/>
-    <mergeCell ref="A10:B10"/>
-    <mergeCell ref="O7:T7"/>
-    <mergeCell ref="V5:AF5"/>
-    <mergeCell ref="V7:AF7"/>
-    <mergeCell ref="D13:AJ13"/>
-    <mergeCell ref="C10:E10"/>
-    <mergeCell ref="C13:C15"/>
-    <mergeCell ref="A7:C7"/>
-    <mergeCell ref="J10:L10"/>
-    <mergeCell ref="AJ14:AJ15"/>
-    <mergeCell ref="Q5:T5"/>
-    <mergeCell ref="D5:M5"/>
-    <mergeCell ref="A23:B23"/>
-    <mergeCell ref="A17:B17"/>
-    <mergeCell ref="A18:B18"/>
-    <mergeCell ref="D7:M7"/>
-    <mergeCell ref="A19:B19"/>
-    <mergeCell ref="A20:B20"/>
-    <mergeCell ref="A21:B21"/>
-    <mergeCell ref="A22:B22"/>
-    <mergeCell ref="A16:B16"/>
-    <mergeCell ref="A40:C40"/>
-    <mergeCell ref="D40:I40"/>
-    <mergeCell ref="D39:I39"/>
-    <mergeCell ref="A24:B24"/>
-    <mergeCell ref="A30:B30"/>
-    <mergeCell ref="A25:B25"/>
-    <mergeCell ref="A26:B26"/>
-    <mergeCell ref="A27:B27"/>
-    <mergeCell ref="A28:B28"/>
-    <mergeCell ref="A29:B29"/>
-    <mergeCell ref="A31:B31"/>
-    <mergeCell ref="A32:B32"/>
-    <mergeCell ref="A39:C39"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <printOptions horizontalCentered="1"/>
@@ -6278,6 +6268,21 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100615363ACEEE6B944A709FC5E830D8EB7" ma:contentTypeVersion="13" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="d6c7a3079c66bb086b7536931b4c2839">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="48a87fbc-1122-44f2-93f1-d72eaa64fc49" xmlns:ns4="1f35814d-5a13-4e35-8302-a9569db6d944" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="434f7db1c017567e806831a368683dcf" ns3:_="" ns4:_="">
     <xsd:import namespace="48a87fbc-1122-44f2-93f1-d72eaa64fc49"/>
@@ -6500,22 +6505,32 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E8430F91-8599-424E-88AA-E2228D491CF3}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="1f35814d-5a13-4e35-8302-a9569db6d944"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="48a87fbc-1122-44f2-93f1-d72eaa64fc49"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B275E3D4-4296-4547-B196-BDA72E71ECC6}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E677A296-6B6F-428B-A7EC-C966B8C36EB2}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -6532,29 +6547,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B275E3D4-4296-4547-B196-BDA72E71ECC6}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E8430F91-8599-424E-88AA-E2228D491CF3}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="1f35814d-5a13-4e35-8302-a9569db6d944"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="48a87fbc-1122-44f2-93f1-d72eaa64fc49"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Update: ../Samples/GEC template timesheet Single 08.08.2025.xlsx
</commit_message>
<xml_diff>
--- a/Samples/GEC template timesheet Single 08.08.2025.xlsx
+++ b/Samples/GEC template timesheet Single 08.08.2025.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Projects\GEC\Samples\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C6FE9393-97AD-4660-A50B-A2B6AA319200}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{526A88FA-E29F-4C6B-A5A6-45C94076E8CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" tabRatio="836" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -125,7 +125,7 @@
     <t>Spain</t>
   </si>
   <si>
-    <t>Dummy Name 1</t>
+    <t>Employee_1</t>
   </si>
 </sst>
 </file>
@@ -1223,6 +1223,216 @@
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="0" fontId="16" fillId="2" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="30" fillId="0" borderId="27" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="168" fontId="30" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="168" fontId="30" fillId="0" borderId="39" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="165" fontId="21" fillId="0" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="165" fontId="21" fillId="0" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="165" fontId="21" fillId="0" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="21" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="21" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="5" borderId="46" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="5" borderId="47" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="7" borderId="42" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="7" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="7" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="7" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="7" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="7" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="49" fontId="21" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="21" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="21" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="5" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="5" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="5" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="26" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="26" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="26" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="7" borderId="43" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="7" borderId="44" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="16" fillId="5" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="16" fillId="5" borderId="44" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="45" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="4" borderId="42" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="4" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="4" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="46" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="2" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="2" borderId="48" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1243,26 +1453,6 @@
       <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left"/>
-      <protection locked="0"/>
-    </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left"/>
       <protection locked="0"/>
@@ -1340,196 +1530,6 @@
       <protection locked="0"/>
     </xf>
     <xf numFmtId="165" fontId="34" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="45" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="4" borderId="42" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="4" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="4" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="46" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="2" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="2" borderId="48" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="5" borderId="46" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="5" borderId="47" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="7" borderId="42" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="7" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="7" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="7" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="7" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="7" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="49" fontId="21" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="49" fontId="21" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="49" fontId="21" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="5" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="5" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="5" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="26" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="26" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="26" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="7" borderId="43" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="7" borderId="44" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="16" fillId="5" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="16" fillId="5" borderId="44" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="49" fontId="21" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="21" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="2" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="30" fillId="0" borderId="27" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="168" fontId="30" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="168" fontId="30" fillId="0" borderId="39" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="165" fontId="21" fillId="0" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="165" fontId="21" fillId="0" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="165" fontId="21" fillId="0" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
@@ -3798,46 +3798,46 @@
       <c r="AO4" s="10"/>
     </row>
     <row r="5" spans="1:53" s="14" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.6">
-      <c r="A5" s="123" t="s">
+      <c r="A5" s="94" t="s">
         <v>14</v>
       </c>
-      <c r="B5" s="123"/>
-      <c r="C5" s="124"/>
-      <c r="D5" s="149" t="s">
+      <c r="B5" s="94"/>
+      <c r="C5" s="95"/>
+      <c r="D5" s="120" t="s">
         <v>33</v>
       </c>
-      <c r="E5" s="150"/>
-      <c r="F5" s="150"/>
-      <c r="G5" s="150"/>
-      <c r="H5" s="150"/>
-      <c r="I5" s="150"/>
-      <c r="J5" s="150"/>
-      <c r="K5" s="150"/>
-      <c r="L5" s="150"/>
-      <c r="M5" s="151"/>
+      <c r="E5" s="121"/>
+      <c r="F5" s="121"/>
+      <c r="G5" s="121"/>
+      <c r="H5" s="121"/>
+      <c r="I5" s="121"/>
+      <c r="J5" s="121"/>
+      <c r="K5" s="121"/>
+      <c r="L5" s="121"/>
+      <c r="M5" s="122"/>
       <c r="N5" s="54"/>
       <c r="O5" s="54"/>
       <c r="P5" s="54"/>
-      <c r="Q5" s="133" t="s">
+      <c r="Q5" s="104" t="s">
         <v>15</v>
       </c>
-      <c r="R5" s="133"/>
-      <c r="S5" s="133"/>
-      <c r="T5" s="133"/>
+      <c r="R5" s="104"/>
+      <c r="S5" s="104"/>
+      <c r="T5" s="104"/>
       <c r="U5" s="13"/>
-      <c r="V5" s="134" t="s">
+      <c r="V5" s="105" t="s">
         <v>31</v>
       </c>
-      <c r="W5" s="135"/>
-      <c r="X5" s="135"/>
-      <c r="Y5" s="135"/>
-      <c r="Z5" s="135"/>
-      <c r="AA5" s="135"/>
-      <c r="AB5" s="135"/>
-      <c r="AC5" s="135"/>
-      <c r="AD5" s="135"/>
-      <c r="AE5" s="135"/>
-      <c r="AF5" s="136"/>
+      <c r="W5" s="106"/>
+      <c r="X5" s="106"/>
+      <c r="Y5" s="106"/>
+      <c r="Z5" s="106"/>
+      <c r="AA5" s="106"/>
+      <c r="AB5" s="106"/>
+      <c r="AC5" s="106"/>
+      <c r="AD5" s="106"/>
+      <c r="AE5" s="106"/>
+      <c r="AF5" s="107"/>
       <c r="AG5" s="58"/>
       <c r="AH5" s="58"/>
       <c r="AI5" s="58"/>
@@ -3891,46 +3891,46 @@
       <c r="AY6" s="17"/>
     </row>
     <row r="7" spans="1:53" s="14" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.65">
-      <c r="A7" s="123" t="s">
+      <c r="A7" s="94" t="s">
         <v>19</v>
       </c>
-      <c r="B7" s="123"/>
-      <c r="C7" s="124"/>
-      <c r="D7" s="152" t="s">
+      <c r="B7" s="94"/>
+      <c r="C7" s="95"/>
+      <c r="D7" s="86" t="s">
         <v>25</v>
       </c>
-      <c r="E7" s="153"/>
-      <c r="F7" s="153"/>
-      <c r="G7" s="153"/>
-      <c r="H7" s="153"/>
-      <c r="I7" s="154"/>
-      <c r="J7" s="154"/>
-      <c r="K7" s="154"/>
-      <c r="L7" s="154"/>
-      <c r="M7" s="155"/>
+      <c r="E7" s="87"/>
+      <c r="F7" s="87"/>
+      <c r="G7" s="87"/>
+      <c r="H7" s="87"/>
+      <c r="I7" s="88"/>
+      <c r="J7" s="88"/>
+      <c r="K7" s="88"/>
+      <c r="L7" s="88"/>
+      <c r="M7" s="89"/>
       <c r="N7" s="54"/>
-      <c r="O7" s="133" t="s">
+      <c r="O7" s="104" t="s">
         <v>20</v>
       </c>
-      <c r="P7" s="133"/>
-      <c r="Q7" s="133"/>
-      <c r="R7" s="133"/>
-      <c r="S7" s="133"/>
-      <c r="T7" s="133"/>
+      <c r="P7" s="104"/>
+      <c r="Q7" s="104"/>
+      <c r="R7" s="104"/>
+      <c r="S7" s="104"/>
+      <c r="T7" s="104"/>
       <c r="U7" s="13"/>
-      <c r="V7" s="134" t="s">
+      <c r="V7" s="105" t="s">
         <v>26</v>
       </c>
-      <c r="W7" s="135"/>
-      <c r="X7" s="135"/>
-      <c r="Y7" s="135"/>
-      <c r="Z7" s="135"/>
-      <c r="AA7" s="135"/>
-      <c r="AB7" s="135"/>
-      <c r="AC7" s="135"/>
-      <c r="AD7" s="135"/>
-      <c r="AE7" s="135"/>
-      <c r="AF7" s="136"/>
+      <c r="W7" s="106"/>
+      <c r="X7" s="106"/>
+      <c r="Y7" s="106"/>
+      <c r="Z7" s="106"/>
+      <c r="AA7" s="106"/>
+      <c r="AB7" s="106"/>
+      <c r="AC7" s="106"/>
+      <c r="AD7" s="106"/>
+      <c r="AE7" s="106"/>
+      <c r="AF7" s="107"/>
       <c r="AG7" s="58"/>
       <c r="AH7" s="58"/>
       <c r="AI7" s="58"/>
@@ -3985,8 +3985,8 @@
       <c r="AR8" s="17"/>
     </row>
     <row r="9" spans="1:53" s="14" customFormat="1" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.6">
-      <c r="A9" s="131"/>
-      <c r="B9" s="131"/>
+      <c r="A9" s="102"/>
+      <c r="B9" s="102"/>
       <c r="C9" s="25"/>
       <c r="D9" s="54"/>
       <c r="E9" s="54"/>
@@ -4026,21 +4026,21 @@
       <c r="AR9" s="17"/>
     </row>
     <row r="10" spans="1:53" s="14" customFormat="1" ht="26" thickBot="1" x14ac:dyDescent="0.6">
-      <c r="A10" s="132" t="s">
+      <c r="A10" s="103" t="s">
         <v>2</v>
       </c>
-      <c r="B10" s="132"/>
-      <c r="C10" s="140">
+      <c r="B10" s="103"/>
+      <c r="C10" s="111">
         <v>45870</v>
       </c>
-      <c r="D10" s="141"/>
-      <c r="E10" s="142"/>
+      <c r="D10" s="112"/>
+      <c r="E10" s="113"/>
       <c r="G10" s="12"/>
       <c r="H10"/>
       <c r="I10" s="26"/>
-      <c r="J10" s="146"/>
-      <c r="K10" s="146"/>
-      <c r="L10" s="146"/>
+      <c r="J10" s="117"/>
+      <c r="K10" s="117"/>
+      <c r="L10" s="117"/>
       <c r="M10" s="27"/>
       <c r="N10" s="27"/>
       <c r="O10" s="27"/>
@@ -4137,55 +4137,55 @@
       <c r="AU12" s="35"/>
     </row>
     <row r="13" spans="1:53" s="37" customFormat="1" ht="33" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="125" t="s">
+      <c r="A13" s="96" t="s">
         <v>21</v>
       </c>
-      <c r="B13" s="126"/>
-      <c r="C13" s="143" t="s">
+      <c r="B13" s="97"/>
+      <c r="C13" s="114" t="s">
         <v>22</v>
       </c>
-      <c r="D13" s="137" t="s">
+      <c r="D13" s="108" t="s">
         <v>4</v>
       </c>
-      <c r="E13" s="138"/>
-      <c r="F13" s="138"/>
-      <c r="G13" s="138"/>
-      <c r="H13" s="138"/>
-      <c r="I13" s="138"/>
-      <c r="J13" s="138"/>
-      <c r="K13" s="138"/>
-      <c r="L13" s="138"/>
-      <c r="M13" s="138"/>
-      <c r="N13" s="138"/>
-      <c r="O13" s="138"/>
-      <c r="P13" s="138"/>
-      <c r="Q13" s="138"/>
-      <c r="R13" s="138"/>
-      <c r="S13" s="138"/>
-      <c r="T13" s="138"/>
-      <c r="U13" s="138"/>
-      <c r="V13" s="138"/>
-      <c r="W13" s="138"/>
-      <c r="X13" s="138"/>
-      <c r="Y13" s="138"/>
-      <c r="Z13" s="138"/>
-      <c r="AA13" s="138"/>
-      <c r="AB13" s="138"/>
-      <c r="AC13" s="138"/>
-      <c r="AD13" s="138"/>
-      <c r="AE13" s="138"/>
-      <c r="AF13" s="138"/>
-      <c r="AG13" s="138"/>
-      <c r="AH13" s="138"/>
-      <c r="AI13" s="138"/>
-      <c r="AJ13" s="139"/>
+      <c r="E13" s="109"/>
+      <c r="F13" s="109"/>
+      <c r="G13" s="109"/>
+      <c r="H13" s="109"/>
+      <c r="I13" s="109"/>
+      <c r="J13" s="109"/>
+      <c r="K13" s="109"/>
+      <c r="L13" s="109"/>
+      <c r="M13" s="109"/>
+      <c r="N13" s="109"/>
+      <c r="O13" s="109"/>
+      <c r="P13" s="109"/>
+      <c r="Q13" s="109"/>
+      <c r="R13" s="109"/>
+      <c r="S13" s="109"/>
+      <c r="T13" s="109"/>
+      <c r="U13" s="109"/>
+      <c r="V13" s="109"/>
+      <c r="W13" s="109"/>
+      <c r="X13" s="109"/>
+      <c r="Y13" s="109"/>
+      <c r="Z13" s="109"/>
+      <c r="AA13" s="109"/>
+      <c r="AB13" s="109"/>
+      <c r="AC13" s="109"/>
+      <c r="AD13" s="109"/>
+      <c r="AE13" s="109"/>
+      <c r="AF13" s="109"/>
+      <c r="AG13" s="109"/>
+      <c r="AH13" s="109"/>
+      <c r="AI13" s="109"/>
+      <c r="AJ13" s="110"/>
       <c r="AK13" s="36"/>
       <c r="AL13" s="36"/>
     </row>
     <row r="14" spans="1:53" s="37" customFormat="1" ht="26.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A14" s="127"/>
-      <c r="B14" s="128"/>
-      <c r="C14" s="144"/>
+      <c r="A14" s="98"/>
+      <c r="B14" s="99"/>
+      <c r="C14" s="115"/>
       <c r="D14" s="59" t="str">
         <f t="shared" ref="D14:AG14" si="0">TEXT(D15, "ddd")</f>
         <v>Fri</v>
@@ -4309,10 +4309,10 @@
       <c r="AH14" s="60" t="s">
         <v>30</v>
       </c>
-      <c r="AI14" s="121" t="s">
+      <c r="AI14" s="92" t="s">
         <v>23</v>
       </c>
-      <c r="AJ14" s="147" t="s">
+      <c r="AJ14" s="118" t="s">
         <v>5</v>
       </c>
       <c r="AK14" s="36"/>
@@ -4334,9 +4334,9 @@
       <c r="BA14" s="36"/>
     </row>
     <row r="15" spans="1:53" s="38" customFormat="1" ht="26.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A15" s="129"/>
-      <c r="B15" s="130"/>
-      <c r="C15" s="145"/>
+      <c r="A15" s="100"/>
+      <c r="B15" s="101"/>
+      <c r="C15" s="116"/>
       <c r="D15" s="61">
         <f>C10</f>
         <v>45870</v>
@@ -4461,18 +4461,18 @@
         <f t="shared" si="4"/>
         <v>45900</v>
       </c>
-      <c r="AI15" s="122"/>
-      <c r="AJ15" s="148"/>
+      <c r="AI15" s="93"/>
+      <c r="AJ15" s="119"/>
       <c r="AR15" s="8"/>
       <c r="AS15" s="8"/>
       <c r="AT15" s="10"/>
       <c r="AU15" s="10"/>
     </row>
     <row r="16" spans="1:53" s="39" customFormat="1" ht="26.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A16" s="156" t="s">
+      <c r="A16" s="90" t="s">
         <v>32</v>
       </c>
-      <c r="B16" s="157"/>
+      <c r="B16" s="91"/>
       <c r="C16" s="3" t="s">
         <v>27</v>
       </c>
@@ -4552,10 +4552,10 @@
       <c r="AU16" s="10"/>
     </row>
     <row r="17" spans="1:47" s="39" customFormat="1" ht="26.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A17" s="82" t="s">
+      <c r="A17" s="84" t="s">
         <v>31</v>
       </c>
-      <c r="B17" s="83"/>
+      <c r="B17" s="85"/>
       <c r="C17" s="3" t="s">
         <v>28</v>
       </c>
@@ -4621,10 +4621,10 @@
       <c r="AU17" s="10"/>
     </row>
     <row r="18" spans="1:47" s="39" customFormat="1" ht="26.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A18" s="82" t="s">
+      <c r="A18" s="84" t="s">
         <v>31</v>
       </c>
-      <c r="B18" s="83"/>
+      <c r="B18" s="85"/>
       <c r="C18" s="3" t="s">
         <v>29</v>
       </c>
@@ -4678,8 +4678,8 @@
       <c r="AU18" s="10"/>
     </row>
     <row r="19" spans="1:47" s="39" customFormat="1" ht="26.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A19" s="82"/>
-      <c r="B19" s="83"/>
+      <c r="A19" s="84"/>
+      <c r="B19" s="85"/>
       <c r="C19" s="3"/>
       <c r="D19" s="57"/>
       <c r="E19" s="57"/>
@@ -4723,8 +4723,8 @@
       <c r="AU19" s="10"/>
     </row>
     <row r="20" spans="1:47" s="39" customFormat="1" ht="26.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A20" s="82"/>
-      <c r="B20" s="83"/>
+      <c r="A20" s="84"/>
+      <c r="B20" s="85"/>
       <c r="C20" s="3"/>
       <c r="D20" s="57"/>
       <c r="E20" s="57"/>
@@ -4768,8 +4768,8 @@
       <c r="AU20" s="10"/>
     </row>
     <row r="21" spans="1:47" s="39" customFormat="1" ht="26.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A21" s="82"/>
-      <c r="B21" s="83"/>
+      <c r="A21" s="84"/>
+      <c r="B21" s="85"/>
       <c r="C21" s="3"/>
       <c r="D21" s="57"/>
       <c r="E21" s="57"/>
@@ -4813,8 +4813,8 @@
       <c r="AU21" s="10"/>
     </row>
     <row r="22" spans="1:47" s="39" customFormat="1" ht="26.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A22" s="82"/>
-      <c r="B22" s="83"/>
+      <c r="A22" s="84"/>
+      <c r="B22" s="85"/>
       <c r="C22" s="3"/>
       <c r="D22" s="57"/>
       <c r="E22" s="57"/>
@@ -4858,8 +4858,8 @@
       <c r="AU22" s="10"/>
     </row>
     <row r="23" spans="1:47" s="39" customFormat="1" ht="26.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A23" s="82"/>
-      <c r="B23" s="83"/>
+      <c r="A23" s="84"/>
+      <c r="B23" s="85"/>
       <c r="C23" s="3"/>
       <c r="D23" s="57"/>
       <c r="E23" s="57"/>
@@ -4903,8 +4903,8 @@
       <c r="AU23" s="10"/>
     </row>
     <row r="24" spans="1:47" s="39" customFormat="1" ht="26.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A24" s="82"/>
-      <c r="B24" s="83"/>
+      <c r="A24" s="84"/>
+      <c r="B24" s="85"/>
       <c r="C24" s="3"/>
       <c r="D24" s="57"/>
       <c r="E24" s="57"/>
@@ -4948,8 +4948,8 @@
       <c r="AU24" s="10"/>
     </row>
     <row r="25" spans="1:47" s="39" customFormat="1" ht="26.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A25" s="82"/>
-      <c r="B25" s="83"/>
+      <c r="A25" s="84"/>
+      <c r="B25" s="85"/>
       <c r="C25" s="3"/>
       <c r="D25" s="57"/>
       <c r="E25" s="57"/>
@@ -4993,8 +4993,8 @@
       <c r="AU25" s="10"/>
     </row>
     <row r="26" spans="1:47" s="39" customFormat="1" ht="26.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A26" s="82"/>
-      <c r="B26" s="83"/>
+      <c r="A26" s="84"/>
+      <c r="B26" s="85"/>
       <c r="C26" s="3"/>
       <c r="D26" s="57"/>
       <c r="E26" s="57"/>
@@ -5038,8 +5038,8 @@
       <c r="AU26" s="10"/>
     </row>
     <row r="27" spans="1:47" s="39" customFormat="1" ht="26.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A27" s="82"/>
-      <c r="B27" s="83"/>
+      <c r="A27" s="84"/>
+      <c r="B27" s="85"/>
       <c r="C27" s="3"/>
       <c r="D27" s="57"/>
       <c r="E27" s="57"/>
@@ -5083,8 +5083,8 @@
       <c r="AU27" s="10"/>
     </row>
     <row r="28" spans="1:47" s="39" customFormat="1" ht="26.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A28" s="82"/>
-      <c r="B28" s="83"/>
+      <c r="A28" s="84"/>
+      <c r="B28" s="85"/>
       <c r="C28" s="3"/>
       <c r="D28" s="57"/>
       <c r="E28" s="57"/>
@@ -5128,8 +5128,8 @@
       <c r="AU28" s="10"/>
     </row>
     <row r="29" spans="1:47" s="39" customFormat="1" ht="26.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A29" s="82"/>
-      <c r="B29" s="83"/>
+      <c r="A29" s="84"/>
+      <c r="B29" s="85"/>
       <c r="C29" s="3"/>
       <c r="D29" s="57"/>
       <c r="E29" s="57"/>
@@ -5173,8 +5173,8 @@
       <c r="AU29" s="10"/>
     </row>
     <row r="30" spans="1:47" s="39" customFormat="1" ht="26.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A30" s="82"/>
-      <c r="B30" s="83"/>
+      <c r="A30" s="84"/>
+      <c r="B30" s="85"/>
       <c r="C30" s="3"/>
       <c r="D30" s="57"/>
       <c r="E30" s="57"/>
@@ -5218,8 +5218,8 @@
       <c r="AU30" s="10"/>
     </row>
     <row r="31" spans="1:47" s="39" customFormat="1" ht="26.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A31" s="82"/>
-      <c r="B31" s="83"/>
+      <c r="A31" s="84"/>
+      <c r="B31" s="85"/>
       <c r="C31" s="3"/>
       <c r="D31" s="1"/>
       <c r="E31" s="1"/>
@@ -5263,8 +5263,8 @@
       <c r="AU31" s="10"/>
     </row>
     <row r="32" spans="1:47" s="40" customFormat="1" ht="26.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A32" s="82"/>
-      <c r="B32" s="83"/>
+      <c r="A32" s="84"/>
+      <c r="B32" s="85"/>
       <c r="C32" s="3"/>
       <c r="D32" s="1"/>
       <c r="E32" s="1"/>
@@ -5308,8 +5308,8 @@
       <c r="AU32" s="10"/>
     </row>
     <row r="33" spans="1:47" s="40" customFormat="1" ht="26.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A33" s="82"/>
-      <c r="B33" s="83"/>
+      <c r="A33" s="84"/>
+      <c r="B33" s="85"/>
       <c r="C33" s="3"/>
       <c r="D33" s="1"/>
       <c r="E33" s="1"/>
@@ -5353,8 +5353,8 @@
       <c r="AU33" s="10"/>
     </row>
     <row r="34" spans="1:47" s="40" customFormat="1" ht="26.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A34" s="82"/>
-      <c r="B34" s="83"/>
+      <c r="A34" s="84"/>
+      <c r="B34" s="85"/>
       <c r="C34" s="3"/>
       <c r="D34" s="1"/>
       <c r="E34" s="1"/>
@@ -5398,8 +5398,8 @@
       <c r="AU34" s="10"/>
     </row>
     <row r="35" spans="1:47" s="40" customFormat="1" ht="26.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A35" s="80"/>
-      <c r="B35" s="81"/>
+      <c r="A35" s="142"/>
+      <c r="B35" s="143"/>
       <c r="C35" s="4"/>
       <c r="D35" s="2"/>
       <c r="E35" s="2"/>
@@ -5443,11 +5443,11 @@
       <c r="AU35" s="10"/>
     </row>
     <row r="36" spans="1:47" s="38" customFormat="1" ht="27" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A36" s="77" t="s">
+      <c r="A36" s="139" t="s">
         <v>6</v>
       </c>
-      <c r="B36" s="78"/>
-      <c r="C36" s="79"/>
+      <c r="B36" s="140"/>
+      <c r="C36" s="141"/>
       <c r="D36" s="65">
         <f t="shared" ref="D36:AJ36" si="6">SUM(D16:D35)</f>
         <v>1</v>
@@ -5628,186 +5628,186 @@
       <c r="AU37" s="10"/>
     </row>
     <row r="38" spans="1:47" ht="36.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A38" s="114" t="s">
+      <c r="A38" s="131" t="s">
         <v>7</v>
       </c>
-      <c r="B38" s="115"/>
-      <c r="C38" s="115"/>
-      <c r="D38" s="116"/>
-      <c r="E38" s="117"/>
-      <c r="F38" s="117"/>
-      <c r="G38" s="117"/>
-      <c r="H38" s="117"/>
-      <c r="I38" s="118"/>
-      <c r="J38" s="119" t="s">
+      <c r="B38" s="132"/>
+      <c r="C38" s="132"/>
+      <c r="D38" s="133"/>
+      <c r="E38" s="134"/>
+      <c r="F38" s="134"/>
+      <c r="G38" s="134"/>
+      <c r="H38" s="134"/>
+      <c r="I38" s="135"/>
+      <c r="J38" s="136" t="s">
         <v>16</v>
       </c>
-      <c r="K38" s="119"/>
-      <c r="L38" s="119"/>
-      <c r="M38" s="119"/>
-      <c r="N38" s="120"/>
-      <c r="O38" s="109"/>
-      <c r="P38" s="110"/>
-      <c r="Q38" s="110"/>
-      <c r="R38" s="110"/>
-      <c r="S38" s="110"/>
-      <c r="T38" s="110"/>
-      <c r="U38" s="110"/>
-      <c r="V38" s="110"/>
-      <c r="W38" s="111" t="s">
+      <c r="K38" s="136"/>
+      <c r="L38" s="136"/>
+      <c r="M38" s="136"/>
+      <c r="N38" s="137"/>
+      <c r="O38" s="126"/>
+      <c r="P38" s="127"/>
+      <c r="Q38" s="127"/>
+      <c r="R38" s="127"/>
+      <c r="S38" s="127"/>
+      <c r="T38" s="127"/>
+      <c r="U38" s="127"/>
+      <c r="V38" s="127"/>
+      <c r="W38" s="128" t="s">
         <v>8</v>
       </c>
-      <c r="X38" s="112"/>
-      <c r="Y38" s="112"/>
-      <c r="Z38" s="112"/>
-      <c r="AA38" s="112"/>
-      <c r="AB38" s="112"/>
-      <c r="AC38" s="112"/>
-      <c r="AD38" s="112"/>
-      <c r="AE38" s="112"/>
-      <c r="AF38" s="112"/>
-      <c r="AG38" s="112"/>
-      <c r="AH38" s="112"/>
-      <c r="AI38" s="112"/>
-      <c r="AJ38" s="113"/>
+      <c r="X38" s="129"/>
+      <c r="Y38" s="129"/>
+      <c r="Z38" s="129"/>
+      <c r="AA38" s="129"/>
+      <c r="AB38" s="129"/>
+      <c r="AC38" s="129"/>
+      <c r="AD38" s="129"/>
+      <c r="AE38" s="129"/>
+      <c r="AF38" s="129"/>
+      <c r="AG38" s="129"/>
+      <c r="AH38" s="129"/>
+      <c r="AI38" s="129"/>
+      <c r="AJ38" s="130"/>
       <c r="AQ38" s="8"/>
       <c r="AR38" s="8"/>
       <c r="AS38" s="10"/>
       <c r="AT38" s="10"/>
     </row>
     <row r="39" spans="1:47" ht="36.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A39" s="158" t="s">
+      <c r="A39" s="76" t="s">
         <v>9</v>
       </c>
-      <c r="B39" s="159"/>
-      <c r="C39" s="159"/>
-      <c r="D39" s="163"/>
-      <c r="E39" s="164"/>
-      <c r="F39" s="164"/>
-      <c r="G39" s="164"/>
-      <c r="H39" s="164"/>
-      <c r="I39" s="165"/>
-      <c r="J39" s="101" t="s">
+      <c r="B39" s="77"/>
+      <c r="C39" s="77"/>
+      <c r="D39" s="81"/>
+      <c r="E39" s="82"/>
+      <c r="F39" s="82"/>
+      <c r="G39" s="82"/>
+      <c r="H39" s="82"/>
+      <c r="I39" s="83"/>
+      <c r="J39" s="158" t="s">
         <v>9</v>
       </c>
-      <c r="K39" s="102"/>
-      <c r="L39" s="102"/>
-      <c r="M39" s="102"/>
-      <c r="N39" s="103"/>
-      <c r="O39" s="107"/>
-      <c r="P39" s="108"/>
-      <c r="Q39" s="108"/>
-      <c r="R39" s="108"/>
-      <c r="S39" s="108"/>
-      <c r="T39" s="108"/>
-      <c r="U39" s="108"/>
-      <c r="V39" s="108"/>
-      <c r="W39" s="84"/>
-      <c r="X39" s="85"/>
-      <c r="Y39" s="85"/>
-      <c r="Z39" s="85"/>
-      <c r="AA39" s="85"/>
-      <c r="AB39" s="85"/>
-      <c r="AC39" s="85"/>
-      <c r="AD39" s="85"/>
-      <c r="AE39" s="85"/>
-      <c r="AF39" s="85"/>
-      <c r="AG39" s="85"/>
-      <c r="AH39" s="85"/>
-      <c r="AI39" s="85"/>
-      <c r="AJ39" s="86"/>
+      <c r="K39" s="159"/>
+      <c r="L39" s="159"/>
+      <c r="M39" s="159"/>
+      <c r="N39" s="160"/>
+      <c r="O39" s="164"/>
+      <c r="P39" s="165"/>
+      <c r="Q39" s="165"/>
+      <c r="R39" s="165"/>
+      <c r="S39" s="165"/>
+      <c r="T39" s="165"/>
+      <c r="U39" s="165"/>
+      <c r="V39" s="165"/>
+      <c r="W39" s="123"/>
+      <c r="X39" s="124"/>
+      <c r="Y39" s="124"/>
+      <c r="Z39" s="124"/>
+      <c r="AA39" s="124"/>
+      <c r="AB39" s="124"/>
+      <c r="AC39" s="124"/>
+      <c r="AD39" s="124"/>
+      <c r="AE39" s="124"/>
+      <c r="AF39" s="124"/>
+      <c r="AG39" s="124"/>
+      <c r="AH39" s="124"/>
+      <c r="AI39" s="124"/>
+      <c r="AJ39" s="125"/>
       <c r="AQ39" s="8"/>
       <c r="AR39" s="8"/>
       <c r="AS39" s="10"/>
       <c r="AT39" s="10"/>
     </row>
     <row r="40" spans="1:47" ht="36.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A40" s="158" t="s">
+      <c r="A40" s="76" t="s">
         <v>10</v>
       </c>
-      <c r="B40" s="159"/>
-      <c r="C40" s="159"/>
-      <c r="D40" s="160"/>
-      <c r="E40" s="161"/>
-      <c r="F40" s="161"/>
-      <c r="G40" s="161"/>
-      <c r="H40" s="161"/>
-      <c r="I40" s="162"/>
-      <c r="J40" s="101" t="s">
+      <c r="B40" s="77"/>
+      <c r="C40" s="77"/>
+      <c r="D40" s="78"/>
+      <c r="E40" s="79"/>
+      <c r="F40" s="79"/>
+      <c r="G40" s="79"/>
+      <c r="H40" s="79"/>
+      <c r="I40" s="80"/>
+      <c r="J40" s="158" t="s">
         <v>10</v>
       </c>
-      <c r="K40" s="102"/>
-      <c r="L40" s="102"/>
-      <c r="M40" s="102"/>
-      <c r="N40" s="103"/>
-      <c r="O40" s="104"/>
-      <c r="P40" s="105"/>
-      <c r="Q40" s="105"/>
-      <c r="R40" s="105"/>
-      <c r="S40" s="105"/>
-      <c r="T40" s="105"/>
-      <c r="U40" s="105"/>
-      <c r="V40" s="106"/>
-      <c r="W40" s="84"/>
-      <c r="X40" s="85"/>
-      <c r="Y40" s="85"/>
-      <c r="Z40" s="85"/>
-      <c r="AA40" s="85"/>
-      <c r="AB40" s="85"/>
-      <c r="AC40" s="85"/>
-      <c r="AD40" s="85"/>
-      <c r="AE40" s="85"/>
-      <c r="AF40" s="85"/>
-      <c r="AG40" s="85"/>
-      <c r="AH40" s="85"/>
-      <c r="AI40" s="85"/>
-      <c r="AJ40" s="86"/>
+      <c r="K40" s="159"/>
+      <c r="L40" s="159"/>
+      <c r="M40" s="159"/>
+      <c r="N40" s="160"/>
+      <c r="O40" s="161"/>
+      <c r="P40" s="162"/>
+      <c r="Q40" s="162"/>
+      <c r="R40" s="162"/>
+      <c r="S40" s="162"/>
+      <c r="T40" s="162"/>
+      <c r="U40" s="162"/>
+      <c r="V40" s="163"/>
+      <c r="W40" s="123"/>
+      <c r="X40" s="124"/>
+      <c r="Y40" s="124"/>
+      <c r="Z40" s="124"/>
+      <c r="AA40" s="124"/>
+      <c r="AB40" s="124"/>
+      <c r="AC40" s="124"/>
+      <c r="AD40" s="124"/>
+      <c r="AE40" s="124"/>
+      <c r="AF40" s="124"/>
+      <c r="AG40" s="124"/>
+      <c r="AH40" s="124"/>
+      <c r="AI40" s="124"/>
+      <c r="AJ40" s="125"/>
       <c r="AQ40" s="8"/>
       <c r="AR40" s="8"/>
       <c r="AS40" s="10"/>
       <c r="AT40" s="10"/>
     </row>
     <row r="41" spans="1:47" ht="36.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A41" s="90" t="s">
+      <c r="A41" s="147" t="s">
         <v>11</v>
       </c>
-      <c r="B41" s="91"/>
-      <c r="C41" s="91"/>
-      <c r="D41" s="92"/>
-      <c r="E41" s="93"/>
-      <c r="F41" s="93"/>
-      <c r="G41" s="93"/>
-      <c r="H41" s="93"/>
-      <c r="I41" s="94"/>
-      <c r="J41" s="98" t="s">
+      <c r="B41" s="148"/>
+      <c r="C41" s="148"/>
+      <c r="D41" s="149"/>
+      <c r="E41" s="150"/>
+      <c r="F41" s="150"/>
+      <c r="G41" s="150"/>
+      <c r="H41" s="150"/>
+      <c r="I41" s="151"/>
+      <c r="J41" s="155" t="s">
         <v>11</v>
       </c>
-      <c r="K41" s="99"/>
-      <c r="L41" s="99"/>
-      <c r="M41" s="99"/>
-      <c r="N41" s="100"/>
-      <c r="O41" s="95"/>
-      <c r="P41" s="96"/>
-      <c r="Q41" s="96"/>
-      <c r="R41" s="96"/>
-      <c r="S41" s="96"/>
-      <c r="T41" s="96"/>
-      <c r="U41" s="96"/>
-      <c r="V41" s="97"/>
-      <c r="W41" s="87"/>
-      <c r="X41" s="88"/>
-      <c r="Y41" s="88"/>
-      <c r="Z41" s="88"/>
-      <c r="AA41" s="88"/>
-      <c r="AB41" s="88"/>
-      <c r="AC41" s="88"/>
-      <c r="AD41" s="88"/>
-      <c r="AE41" s="88"/>
-      <c r="AF41" s="88"/>
-      <c r="AG41" s="88"/>
-      <c r="AH41" s="88"/>
-      <c r="AI41" s="88"/>
-      <c r="AJ41" s="89"/>
+      <c r="K41" s="156"/>
+      <c r="L41" s="156"/>
+      <c r="M41" s="156"/>
+      <c r="N41" s="157"/>
+      <c r="O41" s="152"/>
+      <c r="P41" s="153"/>
+      <c r="Q41" s="153"/>
+      <c r="R41" s="153"/>
+      <c r="S41" s="153"/>
+      <c r="T41" s="153"/>
+      <c r="U41" s="153"/>
+      <c r="V41" s="154"/>
+      <c r="W41" s="144"/>
+      <c r="X41" s="145"/>
+      <c r="Y41" s="145"/>
+      <c r="Z41" s="145"/>
+      <c r="AA41" s="145"/>
+      <c r="AB41" s="145"/>
+      <c r="AC41" s="145"/>
+      <c r="AD41" s="145"/>
+      <c r="AE41" s="145"/>
+      <c r="AF41" s="145"/>
+      <c r="AG41" s="145"/>
+      <c r="AH41" s="145"/>
+      <c r="AI41" s="145"/>
+      <c r="AJ41" s="146"/>
       <c r="AQ41" s="8"/>
       <c r="AR41" s="8"/>
       <c r="AS41" s="10"/>
@@ -5855,86 +5855,86 @@
       <c r="AT42" s="10"/>
     </row>
     <row r="43" spans="1:47" ht="30.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A43" s="76" t="s">
+      <c r="A43" s="138" t="s">
         <v>12</v>
       </c>
-      <c r="B43" s="76"/>
-      <c r="C43" s="76"/>
-      <c r="D43" s="76"/>
-      <c r="E43" s="76"/>
-      <c r="F43" s="76"/>
-      <c r="G43" s="76"/>
-      <c r="H43" s="76"/>
-      <c r="I43" s="76"/>
-      <c r="J43" s="76"/>
-      <c r="K43" s="76"/>
-      <c r="L43" s="76"/>
-      <c r="M43" s="76"/>
-      <c r="N43" s="76"/>
-      <c r="O43" s="76"/>
-      <c r="P43" s="76"/>
-      <c r="Q43" s="76"/>
-      <c r="R43" s="76"/>
-      <c r="S43" s="76"/>
-      <c r="T43" s="76"/>
-      <c r="U43" s="76"/>
-      <c r="V43" s="76"/>
-      <c r="W43" s="76"/>
-      <c r="X43" s="76"/>
-      <c r="Y43" s="76"/>
-      <c r="Z43" s="76"/>
-      <c r="AA43" s="76"/>
-      <c r="AB43" s="76"/>
-      <c r="AC43" s="76"/>
-      <c r="AD43" s="76"/>
-      <c r="AE43" s="76"/>
-      <c r="AF43" s="76"/>
-      <c r="AG43" s="76"/>
-      <c r="AH43" s="76"/>
-      <c r="AI43" s="76"/>
-      <c r="AJ43" s="76"/>
+      <c r="B43" s="138"/>
+      <c r="C43" s="138"/>
+      <c r="D43" s="138"/>
+      <c r="E43" s="138"/>
+      <c r="F43" s="138"/>
+      <c r="G43" s="138"/>
+      <c r="H43" s="138"/>
+      <c r="I43" s="138"/>
+      <c r="J43" s="138"/>
+      <c r="K43" s="138"/>
+      <c r="L43" s="138"/>
+      <c r="M43" s="138"/>
+      <c r="N43" s="138"/>
+      <c r="O43" s="138"/>
+      <c r="P43" s="138"/>
+      <c r="Q43" s="138"/>
+      <c r="R43" s="138"/>
+      <c r="S43" s="138"/>
+      <c r="T43" s="138"/>
+      <c r="U43" s="138"/>
+      <c r="V43" s="138"/>
+      <c r="W43" s="138"/>
+      <c r="X43" s="138"/>
+      <c r="Y43" s="138"/>
+      <c r="Z43" s="138"/>
+      <c r="AA43" s="138"/>
+      <c r="AB43" s="138"/>
+      <c r="AC43" s="138"/>
+      <c r="AD43" s="138"/>
+      <c r="AE43" s="138"/>
+      <c r="AF43" s="138"/>
+      <c r="AG43" s="138"/>
+      <c r="AH43" s="138"/>
+      <c r="AI43" s="138"/>
+      <c r="AJ43" s="138"/>
       <c r="AK43" s="45"/>
       <c r="AL43" s="45"/>
     </row>
     <row r="44" spans="1:47" ht="35.25" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A44" s="76" t="s">
+      <c r="A44" s="138" t="s">
         <v>13</v>
       </c>
-      <c r="B44" s="76"/>
-      <c r="C44" s="76"/>
-      <c r="D44" s="76"/>
-      <c r="E44" s="76"/>
-      <c r="F44" s="76"/>
-      <c r="G44" s="76"/>
-      <c r="H44" s="76"/>
-      <c r="I44" s="76"/>
-      <c r="J44" s="76"/>
-      <c r="K44" s="76"/>
-      <c r="L44" s="76"/>
-      <c r="M44" s="76"/>
-      <c r="N44" s="76"/>
-      <c r="O44" s="76"/>
-      <c r="P44" s="76"/>
-      <c r="Q44" s="76"/>
-      <c r="R44" s="76"/>
-      <c r="S44" s="76"/>
-      <c r="T44" s="76"/>
-      <c r="U44" s="76"/>
-      <c r="V44" s="76"/>
-      <c r="W44" s="76"/>
-      <c r="X44" s="76"/>
-      <c r="Y44" s="76"/>
-      <c r="Z44" s="76"/>
-      <c r="AA44" s="76"/>
-      <c r="AB44" s="76"/>
-      <c r="AC44" s="76"/>
-      <c r="AD44" s="76"/>
-      <c r="AE44" s="76"/>
-      <c r="AF44" s="76"/>
-      <c r="AG44" s="76"/>
-      <c r="AH44" s="76"/>
-      <c r="AI44" s="76"/>
-      <c r="AJ44" s="76"/>
+      <c r="B44" s="138"/>
+      <c r="C44" s="138"/>
+      <c r="D44" s="138"/>
+      <c r="E44" s="138"/>
+      <c r="F44" s="138"/>
+      <c r="G44" s="138"/>
+      <c r="H44" s="138"/>
+      <c r="I44" s="138"/>
+      <c r="J44" s="138"/>
+      <c r="K44" s="138"/>
+      <c r="L44" s="138"/>
+      <c r="M44" s="138"/>
+      <c r="N44" s="138"/>
+      <c r="O44" s="138"/>
+      <c r="P44" s="138"/>
+      <c r="Q44" s="138"/>
+      <c r="R44" s="138"/>
+      <c r="S44" s="138"/>
+      <c r="T44" s="138"/>
+      <c r="U44" s="138"/>
+      <c r="V44" s="138"/>
+      <c r="W44" s="138"/>
+      <c r="X44" s="138"/>
+      <c r="Y44" s="138"/>
+      <c r="Z44" s="138"/>
+      <c r="AA44" s="138"/>
+      <c r="AB44" s="138"/>
+      <c r="AC44" s="138"/>
+      <c r="AD44" s="138"/>
+      <c r="AE44" s="138"/>
+      <c r="AF44" s="138"/>
+      <c r="AG44" s="138"/>
+      <c r="AH44" s="138"/>
+      <c r="AI44" s="138"/>
+      <c r="AJ44" s="138"/>
       <c r="AK44" s="45"/>
       <c r="AL44" s="45"/>
     </row>
@@ -6197,28 +6197,28 @@
     </row>
   </sheetData>
   <mergeCells count="60">
-    <mergeCell ref="A40:C40"/>
-    <mergeCell ref="D40:I40"/>
-    <mergeCell ref="D39:I39"/>
-    <mergeCell ref="A24:B24"/>
-    <mergeCell ref="A30:B30"/>
-    <mergeCell ref="A25:B25"/>
-    <mergeCell ref="A26:B26"/>
-    <mergeCell ref="A27:B27"/>
-    <mergeCell ref="A28:B28"/>
-    <mergeCell ref="A29:B29"/>
-    <mergeCell ref="A31:B31"/>
-    <mergeCell ref="A32:B32"/>
-    <mergeCell ref="A39:C39"/>
-    <mergeCell ref="A23:B23"/>
-    <mergeCell ref="A17:B17"/>
-    <mergeCell ref="A18:B18"/>
-    <mergeCell ref="D7:M7"/>
-    <mergeCell ref="A19:B19"/>
-    <mergeCell ref="A20:B20"/>
-    <mergeCell ref="A21:B21"/>
-    <mergeCell ref="A22:B22"/>
-    <mergeCell ref="A16:B16"/>
+    <mergeCell ref="A43:AJ43"/>
+    <mergeCell ref="A44:AJ44"/>
+    <mergeCell ref="A36:C36"/>
+    <mergeCell ref="A35:B35"/>
+    <mergeCell ref="A33:B33"/>
+    <mergeCell ref="A34:B34"/>
+    <mergeCell ref="W40:AJ40"/>
+    <mergeCell ref="W41:AJ41"/>
+    <mergeCell ref="A41:C41"/>
+    <mergeCell ref="D41:I41"/>
+    <mergeCell ref="O41:V41"/>
+    <mergeCell ref="J41:N41"/>
+    <mergeCell ref="J39:N39"/>
+    <mergeCell ref="J40:N40"/>
+    <mergeCell ref="O40:V40"/>
+    <mergeCell ref="O39:V39"/>
+    <mergeCell ref="W39:AJ39"/>
+    <mergeCell ref="O38:V38"/>
+    <mergeCell ref="W38:AJ38"/>
+    <mergeCell ref="A38:C38"/>
+    <mergeCell ref="D38:I38"/>
+    <mergeCell ref="J38:N38"/>
     <mergeCell ref="AI14:AI15"/>
     <mergeCell ref="A5:C5"/>
     <mergeCell ref="A13:B15"/>
@@ -6235,28 +6235,28 @@
     <mergeCell ref="AJ14:AJ15"/>
     <mergeCell ref="Q5:T5"/>
     <mergeCell ref="D5:M5"/>
-    <mergeCell ref="W39:AJ39"/>
-    <mergeCell ref="O38:V38"/>
-    <mergeCell ref="W38:AJ38"/>
-    <mergeCell ref="A38:C38"/>
-    <mergeCell ref="D38:I38"/>
-    <mergeCell ref="J38:N38"/>
-    <mergeCell ref="A43:AJ43"/>
-    <mergeCell ref="A44:AJ44"/>
-    <mergeCell ref="A36:C36"/>
-    <mergeCell ref="A35:B35"/>
-    <mergeCell ref="A33:B33"/>
-    <mergeCell ref="A34:B34"/>
-    <mergeCell ref="W40:AJ40"/>
-    <mergeCell ref="W41:AJ41"/>
-    <mergeCell ref="A41:C41"/>
-    <mergeCell ref="D41:I41"/>
-    <mergeCell ref="O41:V41"/>
-    <mergeCell ref="J41:N41"/>
-    <mergeCell ref="J39:N39"/>
-    <mergeCell ref="J40:N40"/>
-    <mergeCell ref="O40:V40"/>
-    <mergeCell ref="O39:V39"/>
+    <mergeCell ref="A23:B23"/>
+    <mergeCell ref="A17:B17"/>
+    <mergeCell ref="A18:B18"/>
+    <mergeCell ref="D7:M7"/>
+    <mergeCell ref="A19:B19"/>
+    <mergeCell ref="A20:B20"/>
+    <mergeCell ref="A21:B21"/>
+    <mergeCell ref="A22:B22"/>
+    <mergeCell ref="A16:B16"/>
+    <mergeCell ref="A40:C40"/>
+    <mergeCell ref="D40:I40"/>
+    <mergeCell ref="D39:I39"/>
+    <mergeCell ref="A24:B24"/>
+    <mergeCell ref="A30:B30"/>
+    <mergeCell ref="A25:B25"/>
+    <mergeCell ref="A26:B26"/>
+    <mergeCell ref="A27:B27"/>
+    <mergeCell ref="A28:B28"/>
+    <mergeCell ref="A29:B29"/>
+    <mergeCell ref="A31:B31"/>
+    <mergeCell ref="A32:B32"/>
+    <mergeCell ref="A39:C39"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <printOptions horizontalCentered="1"/>
@@ -6268,21 +6268,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100615363ACEEE6B944A709FC5E830D8EB7" ma:contentTypeVersion="13" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="d6c7a3079c66bb086b7536931b4c2839">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="48a87fbc-1122-44f2-93f1-d72eaa64fc49" xmlns:ns4="1f35814d-5a13-4e35-8302-a9569db6d944" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="434f7db1c017567e806831a368683dcf" ns3:_="" ns4:_="">
     <xsd:import namespace="48a87fbc-1122-44f2-93f1-d72eaa64fc49"/>
@@ -6505,32 +6490,22 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E8430F91-8599-424E-88AA-E2228D491CF3}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="1f35814d-5a13-4e35-8302-a9569db6d944"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="48a87fbc-1122-44f2-93f1-d72eaa64fc49"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B275E3D4-4296-4547-B196-BDA72E71ECC6}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E677A296-6B6F-428B-A7EC-C966B8C36EB2}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -6547,4 +6522,29 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B275E3D4-4296-4547-B196-BDA72E71ECC6}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E8430F91-8599-424E-88AA-E2228D491CF3}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="1f35814d-5a13-4e35-8302-a9569db6d944"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="48a87fbc-1122-44f2-93f1-d72eaa64fc49"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>